<commit_message>
fix(tacografos): entrega del tacografo averiado y achatarramiento vuelven a ser excluyentes
El libro original decidia ambas frases con un unico SI/NO. Se recupera ese
comportamiento: solo se introduce "Se entrega al cliente"; "Se achatarrara" se
calcula como su contrario y queda bloqueado, de modo que el acuse imprime
siempre una sola de las dos lineas.

224 formulas, 0 errores; verificado en los dos sentidos.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TAp9Dxq8XWBh75W4jtVJj4
</commit_message>
<xml_diff>
--- a/docs/plantillas/TACOGRAFOS_documentacion.xlsx
+++ b/docs/plantillas/TACOGRAFOS_documentacion.xlsx
@@ -108,7 +108,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="22">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -146,6 +146,11 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="000000FF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <sz val="10"/>
     </font>
     <font>
@@ -289,95 +294,96 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="justify" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="justify" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="justify" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="justify" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
       <protection locked="0" hidden="0"/>
@@ -1552,21 +1558,20 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>Se achatarrará</t>
-        </is>
-      </c>
-      <c r="B46" s="7" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="C46" s="8">
-        <f>IF(AND($B$28="Intransferibilidad",B46=""),"⚠ Obligatorio","")</f>
-        <v/>
-      </c>
-      <c r="D46" s="2">
-        <f>IF(C46&lt;&gt;"",1,0)</f>
-        <v/>
+          <t>Se achatarrará (excluyente)</t>
+        </is>
+      </c>
+      <c r="B46" s="11">
+        <f>IF(B45="Sí","No",IF(B45="No","Sí",""))</f>
+        <v/>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>automático</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="48">
@@ -1575,7 +1580,7 @@
           <t>Coherencia (UNE 66102:2025)</t>
         </is>
       </c>
-      <c r="B48" s="11">
+      <c r="B48" s="12">
         <f>IF(AND($B$28="Transferencia correcta",OR(B36="No",B37="No")),"⚠ Marcado como transferencia correcta pero el anexo II dice que no se pudo transferir/descargar",IF(AND($B$28="Intransferibilidad",B36="Sí"),"⚠ Marcado como intransferibilidad pero el anexo II dice que sí era posible transferir",""))</f>
         <v/>
       </c>
@@ -1610,7 +1615,7 @@
     <dataValidation sqref="B43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=CONFIGURACION!$B$36:$B$39</formula1>
     </dataValidation>
-    <dataValidation sqref="B10 B21 B34 B35 B36 B37 B40 B45 B46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B10 B21 B34 B35 B36 B37 B40 B45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=CONFIGURACION!$C$40:$C$41</formula1>
     </dataValidation>
     <dataValidation sqref="B20 B26 B27 B39 B41" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Fecha no válida" error="Introduce una fecha real en formato dd/mm/aaaa." type="date" operator="between">
@@ -1642,193 +1647,193 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" s="12">
+      <c r="B1" s="13">
         <f>'CONFIGURACION'!$B$4</f>
         <v/>
       </c>
     </row>
     <row r="2" ht="46" customHeight="1">
-      <c r="B2" s="13" t="inlineStr">
+      <c r="B2" s="14" t="inlineStr">
         <is>
           <t>JUSTIFICANTE PARA AUTORIZAR TODO EL PROCESO DE TRANSFERENCIA, EN EL CAMBIO DE UN TACÓGRAFO DIGITAL CON DESCARGA DE LA MEMORIA INTERNA DEL MISMO.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="14">
+      <c r="B3" s="15">
         <f>"Yo, "&amp;IF('DATOS'!$B$8="","",'DATOS'!$B$8)</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="14">
+      <c r="B4" s="15">
         <f>"con N.I.F. nº: "&amp;IF('DATOS'!$B$9="","",'DATOS'!$B$9)</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="14">
+      <c r="B5" s="15">
         <f>"en representación de la empresa de transportes: "&amp;IF('DATOS'!$B$5="","",'DATOS'!$B$5)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="14">
+      <c r="B6" s="15">
         <f>"propietaria del vehículo matrícula: "&amp;UPPER(IF('DATOS'!$B$12="","",'DATOS'!$B$12))</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="14">
+      <c r="B7" s="15">
         <f>'CONFIGURACION'!$B$44&amp;'CONFIGURACION'!$B$4&amp;","</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="14">
+      <c r="B8" s="15">
         <f>'CONFIGURACION'!$B$45&amp;'CONFIGURACION'!$B$6&amp;'CONFIGURACION'!$B$46&amp;" "&amp;IF('DATOS'!$B$17="","",'DATOS'!$B$17)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="14">
+      <c r="B9" s="15">
         <f>"modelo: "&amp;IF('DATOS'!$B$18="","",'DATOS'!$B$18)&amp;"   y número de serie: "&amp;IF('DATOS'!$B$19="","",'DATOS'!$B$19)</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1">
-      <c r="B10" s="15" t="inlineStr">
+      <c r="B10" s="16" t="inlineStr">
         <is>
           <t>instalado en el vehículo de matrícula indicada arriba, que ha de cambiarse, puede ser correctamente descargado en el contenido de su memoria interna.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="46" customHeight="1">
-      <c r="B11" s="15" t="inlineStr">
+      <c r="B11" s="16" t="inlineStr">
         <is>
           <t>Siendo representante de la empresa propietaria del vehículo o estando autorizado por la Dirección de la misma, doy la indicación y autorizo, al centro técnico de tacógrafos de COMERCIAL SEA, S.A. a la descarga de la mencionada memoria interna del tacógrafo.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="60" customHeight="1">
-      <c r="B12" s="15" t="inlineStr">
+      <c r="B12" s="16" t="inlineStr">
         <is>
           <t>Quedo advertido, en caso de no ser uno de los representantes de dicha empresa, de que debo autorizar todo este proceso habiendo recibido indicación expresa de la Dirección de la misma a actuar en el sentido en el que me manifiesto y que el proceso no tendrá respaldo legal si yo falseo esta autorización.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="60" customHeight="1">
-      <c r="B13" s="15" t="inlineStr">
+      <c r="B13" s="16" t="inlineStr">
         <is>
           <t>Doy la indicación, así mismo, de que los archivos de transferencia originados en la mencionada descarga sean entregados a la empresa propietaria del vehículo a través del medio indicado debajo, de entre las cuatro posibles opciones indicadas en el punto 6 de la disposición adicional primera del Real decreto 125:2017 (señálese la opción que proceda)</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="17" t="inlineStr">
         <is>
           <t>Entrega en mano a una persona designada y autorizada para tal por la empresa propietaria del vehículo de matrícula arriba indicada</t>
         </is>
       </c>
-      <c r="H14" s="17">
+      <c r="H14" s="18">
         <f>IF('DATOS'!$B$43="En mano","X","")</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="16" t="inlineStr">
+      <c r="B15" s="17" t="inlineStr">
         <is>
           <t>Entrega por medios electrónicos (por ejemplo, email)</t>
         </is>
       </c>
-      <c r="H15" s="17">
+      <c r="H15" s="18">
         <f>IF('DATOS'!$B$43="Email","X","")</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="16" t="inlineStr">
+      <c r="B16" s="17" t="inlineStr">
         <is>
           <t>Entrega a través de empresa de mensajería</t>
         </is>
       </c>
-      <c r="H16" s="17">
+      <c r="H16" s="18">
         <f>IF('DATOS'!$B$43="Mensajería","X","")</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="16" t="inlineStr">
+      <c r="B17" s="17" t="inlineStr">
         <is>
           <t>Entrega por correo certificado</t>
         </is>
       </c>
-      <c r="H17" s="17">
+      <c r="H17" s="18">
         <f>IF('DATOS'!$B$43="Correo certificado","X","")</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="46" customHeight="1">
-      <c r="B18" s="18">
+      <c r="B18" s="19">
         <f>'CONFIGURACION'!$B$53</f>
         <v/>
       </c>
     </row>
     <row r="19" ht="32" customHeight="1">
-      <c r="B19" s="18">
+      <c r="B19" s="19">
         <f>'CONFIGURACION'!$B$54</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="32" customHeight="1">
-      <c r="B20" s="18">
+      <c r="B20" s="19">
         <f>'CONFIGURACION'!$B$55</f>
         <v/>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
-      <c r="B22" s="19" t="inlineStr">
+      <c r="B22" s="20" t="inlineStr">
         <is>
           <t>FIRMA DE LA PERSONA QUE AUTORIZA LA DESCARGA Y DA LA INDICACIÓN PARA LA MODALIDAD DE ENTREGA DE LOS ARCHIVOS DE TRANSFERENCIA</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="14">
+      <c r="B23" s="15">
         <f>'CONFIGURACION'!$B$47&amp;'CONFIGURACION'!$B$10&amp;'CONFIGURACION'!$B$48&amp;IF('DATOS'!$B$26="","",RIGHT("0"&amp;DAY('DATOS'!$B$26),2)&amp;"/"&amp;RIGHT("0"&amp;MONTH('DATOS'!$B$26),2)&amp;"/"&amp;YEAR('DATOS'!$B$26))</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="20">
+      <c r="B24" s="21">
         <f>IF('DATOS'!$B$28="Transferencia correcta","","— NO APLICA: esta intervención está marcada como Intransferibilidad —")</f>
         <v/>
       </c>
     </row>
     <row r="25" ht="40" customHeight="1"/>
     <row r="26">
-      <c r="B26" s="21" t="n"/>
-      <c r="F26" s="21" t="n"/>
+      <c r="B26" s="22" t="n"/>
+      <c r="F26" s="22" t="n"/>
     </row>
     <row r="27">
-      <c r="B27" s="22" t="inlineStr">
+      <c r="B27" s="23" t="inlineStr">
         <is>
           <t>Persona que autoriza</t>
         </is>
       </c>
-      <c r="F27" s="22">
+      <c r="F27" s="23">
         <f>"Técnico: "&amp;IF('DATOS'!$B$29="","",'DATOS'!$B$29)</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="F28" s="14">
+      <c r="F28" s="15">
         <f>'CONFIGURACION'!$B$49&amp;'CONFIGURACION'!$B$4</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="23">
+      <c r="B30" s="24">
         <f>"Formato "&amp;'CONFIGURACION'!$B$22&amp;" · Versión "&amp;'CONFIGURACION'!$B$20&amp;" · Edición "&amp;IF('CONFIGURACION'!$B$21="","",RIGHT("0"&amp;DAY('CONFIGURACION'!$B$21),2)&amp;"/"&amp;RIGHT("0"&amp;MONTH('CONFIGURACION'!$B$21),2)&amp;"/"&amp;YEAR('CONFIGURACION'!$B$21))&amp;" · Elaborado: "&amp;'CONFIGURACION'!$B$16&amp;" · Aprobado: "&amp;'CONFIGURACION'!$B$17&amp;" · UNE 66102:2025"</f>
         <v/>
       </c>
@@ -1896,505 +1901,505 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="24" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t>INFORME SOBRE TRANSFERENCIA DE DATOS / CERTIFICADO DE INTRANSFERIBILIDAD</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="25">
+      <c r="A2" s="26">
         <f>"NÚMERO DE INFORME/CERTIFICADO: "&amp;IF('DATOS'!$B$25="","-",'DATOS'!$B$25)</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="26" t="inlineStr">
+      <c r="A4" s="27" t="inlineStr">
         <is>
           <t>DATOS DEL VEHÍCULO Y DE LA EMPRESA</t>
         </is>
       </c>
-      <c r="B4" s="27" t="n"/>
-      <c r="C4" s="27" t="n"/>
-      <c r="D4" s="27" t="n"/>
-      <c r="E4" s="27" t="n"/>
-      <c r="F4" s="27" t="n"/>
-      <c r="G4" s="27" t="n"/>
+      <c r="B4" s="28" t="n"/>
+      <c r="C4" s="28" t="n"/>
+      <c r="D4" s="28" t="n"/>
+      <c r="E4" s="28" t="n"/>
+      <c r="F4" s="28" t="n"/>
+      <c r="G4" s="28" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="28" t="n">
+      <c r="A5" s="29" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>Número de matrícula del vehículo</t>
         </is>
       </c>
-      <c r="E5" s="29">
+      <c r="E5" s="30">
         <f>UPPER(IF('DATOS'!$B$12="","-",'DATOS'!$B$12))</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="28" t="n">
+      <c r="A6" s="29" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="17" t="inlineStr">
         <is>
           <t>Número de bastidor del vehículo</t>
         </is>
       </c>
-      <c r="E6" s="29">
+      <c r="E6" s="30">
         <f>IF('DATOS'!$B$13="","-",'DATOS'!$B$13)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="28" t="n">
+      <c r="A7" s="29" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>Fabricante del vehículo</t>
         </is>
       </c>
-      <c r="E7" s="29">
+      <c r="E7" s="30">
         <f>IF('DATOS'!$B$14="","-",'DATOS'!$B$14)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="28" t="n">
+      <c r="A8" s="29" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>Modelo del vehículo</t>
         </is>
       </c>
-      <c r="E8" s="29">
+      <c r="E8" s="30">
         <f>IF('DATOS'!$B$15="","-",'DATOS'!$B$15)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="28" t="n">
+      <c r="A9" s="29" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="16" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t>Nombre de la empresa de transportes</t>
         </is>
       </c>
-      <c r="E9" s="29">
+      <c r="E9" s="30">
         <f>IF('DATOS'!$B$5="","-",'DATOS'!$B$5)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="28" t="n">
+      <c r="A10" s="29" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="16" t="inlineStr">
+      <c r="B10" s="17" t="inlineStr">
         <is>
           <t>Dirección de la empresa de transportes</t>
         </is>
       </c>
-      <c r="E10" s="29">
+      <c r="E10" s="30">
         <f>IF('DATOS'!$B$6="","-",'DATOS'!$B$6)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="28" t="n">
+      <c r="A11" s="29" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>Detalles de la tarjeta de empresa</t>
         </is>
       </c>
-      <c r="E11" s="29">
+      <c r="E11" s="30">
         <f>IF('DATOS'!$B$7="","-",'DATOS'!$B$7)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="26" t="inlineStr">
+      <c r="A12" s="27" t="inlineStr">
         <is>
           <t>DATOS DEL CENTRO TÉCNICO</t>
         </is>
       </c>
-      <c r="B12" s="27" t="n"/>
-      <c r="C12" s="27" t="n"/>
-      <c r="D12" s="27" t="n"/>
-      <c r="E12" s="27" t="n"/>
-      <c r="F12" s="27" t="n"/>
-      <c r="G12" s="27" t="n"/>
+      <c r="B12" s="28" t="n"/>
+      <c r="C12" s="28" t="n"/>
+      <c r="D12" s="28" t="n"/>
+      <c r="E12" s="28" t="n"/>
+      <c r="F12" s="28" t="n"/>
+      <c r="G12" s="28" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="28" t="n">
+      <c r="A13" s="29" t="n">
         <v>8</v>
       </c>
-      <c r="B13" s="16" t="inlineStr">
+      <c r="B13" s="17" t="inlineStr">
         <is>
           <t>Nombre del centro técnico</t>
         </is>
       </c>
-      <c r="E13" s="29">
+      <c r="E13" s="30">
         <f>'CONFIGURACION'!$B$4&amp;" — "&amp;'CONFIGURACION'!$B$5</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="28" t="n">
+      <c r="A14" s="29" t="n">
         <v>9</v>
       </c>
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="17" t="inlineStr">
         <is>
           <t>Dirección del centro técnico</t>
         </is>
       </c>
-      <c r="E14" s="29">
+      <c r="E14" s="30">
         <f>'CONFIGURACION'!$B$7&amp;", "&amp;'CONFIGURACION'!$B$8&amp;", "&amp;'CONFIGURACION'!$B$9</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="28" t="n">
+      <c r="A15" s="29" t="n">
         <v>10</v>
       </c>
-      <c r="B15" s="16" t="inlineStr">
+      <c r="B15" s="17" t="inlineStr">
         <is>
           <t>Contraseña del centro técnico</t>
         </is>
       </c>
-      <c r="E15" s="29">
+      <c r="E15" s="30">
         <f>'CONFIGURACION'!$B$6</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="28" t="n">
+      <c r="A16" s="29" t="n">
         <v>11</v>
       </c>
-      <c r="B16" s="16" t="inlineStr">
+      <c r="B16" s="17" t="inlineStr">
         <is>
           <t>Detalles de la tarjeta del centro técnico</t>
         </is>
       </c>
-      <c r="E16" s="29">
+      <c r="E16" s="30">
         <f>IF('DATOS'!$B$30="","-",'DATOS'!$B$30)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="28" t="n">
+      <c r="A17" s="29" t="n">
         <v>12</v>
       </c>
-      <c r="B17" s="16" t="inlineStr">
+      <c r="B17" s="17" t="inlineStr">
         <is>
           <t>Nombre del técnico que ha intervenido y firma</t>
         </is>
       </c>
-      <c r="E17" s="29">
+      <c r="E17" s="30">
         <f>IF('DATOS'!$B$29="","-",'DATOS'!$B$29)</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="26" t="inlineStr">
+      <c r="A18" s="27" t="inlineStr">
         <is>
           <t>DATOS DE LA UNIDAD INSTALADA EN EL VEHÍCULO</t>
         </is>
       </c>
-      <c r="B18" s="27" t="n"/>
-      <c r="C18" s="27" t="n"/>
-      <c r="D18" s="27" t="n"/>
-      <c r="E18" s="27" t="n"/>
-      <c r="F18" s="27" t="n"/>
-      <c r="G18" s="27" t="n"/>
+      <c r="B18" s="28" t="n"/>
+      <c r="C18" s="28" t="n"/>
+      <c r="D18" s="28" t="n"/>
+      <c r="E18" s="28" t="n"/>
+      <c r="F18" s="28" t="n"/>
+      <c r="G18" s="28" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="28" t="n">
+      <c r="A19" s="29" t="n">
         <v>13</v>
       </c>
-      <c r="B19" s="16" t="inlineStr">
+      <c r="B19" s="17" t="inlineStr">
         <is>
           <t>Nombre del fabricante del tacógrafo</t>
         </is>
       </c>
-      <c r="E19" s="29">
+      <c r="E19" s="30">
         <f>IF('DATOS'!$B$17="","-",'DATOS'!$B$17)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="28" t="n">
+      <c r="A20" s="29" t="n">
         <v>14</v>
       </c>
-      <c r="B20" s="16" t="inlineStr">
+      <c r="B20" s="17" t="inlineStr">
         <is>
           <t>Modelo de la unidad</t>
         </is>
       </c>
-      <c r="E20" s="29">
+      <c r="E20" s="30">
         <f>IF('DATOS'!$B$18="","-",'DATOS'!$B$18)</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="28" t="n">
+      <c r="A21" s="29" t="n">
         <v>15</v>
       </c>
-      <c r="B21" s="16" t="inlineStr">
+      <c r="B21" s="17" t="inlineStr">
         <is>
           <t>Número de serie de la unidad</t>
         </is>
       </c>
-      <c r="E21" s="29">
+      <c r="E21" s="30">
         <f>IF('DATOS'!$B$19="","-",'DATOS'!$B$19)</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="28" t="n">
+      <c r="A22" s="29" t="n">
         <v>16</v>
       </c>
-      <c r="B22" s="16" t="inlineStr">
+      <c r="B22" s="17" t="inlineStr">
         <is>
           <t>Fecha de fabricación de la unidad</t>
         </is>
       </c>
-      <c r="E22" s="29">
+      <c r="E22" s="30">
         <f>IF('DATOS'!$B$20="","-",IF('DATOS'!$B$20="","",RIGHT("0"&amp;DAY('DATOS'!$B$20),2)&amp;"/"&amp;RIGHT("0"&amp;MONTH('DATOS'!$B$20),2)&amp;"/"&amp;YEAR('DATOS'!$B$20)))</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="28" t="n">
+      <c r="A23" s="29" t="n">
         <v>17</v>
       </c>
-      <c r="B23" s="16" t="inlineStr">
+      <c r="B23" s="17" t="inlineStr">
         <is>
           <t>Situación de la unidad en la cabina</t>
         </is>
       </c>
-      <c r="E23" s="29">
+      <c r="E23" s="30">
         <f>IF('DATOS'!$B$21="","-",'DATOS'!$B$21)</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="28" t="n">
+      <c r="A24" s="29" t="n">
         <v>18</v>
       </c>
-      <c r="B24" s="16" t="inlineStr">
+      <c r="B24" s="17" t="inlineStr">
         <is>
           <t>Marca de homologación de la unidad</t>
         </is>
       </c>
-      <c r="E24" s="29">
+      <c r="E24" s="30">
         <f>IF('DATOS'!$B$22="","-",'DATOS'!$B$22)</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="28" t="n">
+      <c r="A25" s="29" t="n">
         <v>19</v>
       </c>
-      <c r="B25" s="16" t="inlineStr">
+      <c r="B25" s="17" t="inlineStr">
         <is>
           <t>Visibilidad de la placa (Req 169/170)</t>
         </is>
       </c>
-      <c r="E25" s="29">
+      <c r="E25" s="30">
         <f>IF('DATOS'!$B$23="","-",'DATOS'!$B$23)</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="26" t="inlineStr">
+      <c r="A26" s="27" t="inlineStr">
         <is>
           <t>DETALLES DE LA TRANSFERENCIA</t>
         </is>
       </c>
-      <c r="B26" s="27" t="n"/>
-      <c r="C26" s="27" t="n"/>
-      <c r="D26" s="27" t="n"/>
-      <c r="E26" s="27" t="n"/>
-      <c r="F26" s="27" t="n"/>
-      <c r="G26" s="27" t="n"/>
+      <c r="B26" s="28" t="n"/>
+      <c r="C26" s="28" t="n"/>
+      <c r="D26" s="28" t="n"/>
+      <c r="E26" s="28" t="n"/>
+      <c r="F26" s="28" t="n"/>
+      <c r="G26" s="28" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="28" t="n">
+      <c r="A27" s="29" t="n">
         <v>20</v>
       </c>
-      <c r="B27" s="16" t="inlineStr">
+      <c r="B27" s="17" t="inlineStr">
         <is>
           <t>¿Se ven los datos en pantalla?</t>
         </is>
       </c>
-      <c r="E27" s="29">
+      <c r="E27" s="30">
         <f>IF('DATOS'!$B$34="","-",'DATOS'!$B$34)</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="28" t="n">
+      <c r="A28" s="29" t="n">
         <v>21</v>
       </c>
-      <c r="B28" s="16" t="inlineStr">
+      <c r="B28" s="17" t="inlineStr">
         <is>
           <t>¿Era posible imprimir los datos?</t>
         </is>
       </c>
-      <c r="E28" s="29">
+      <c r="E28" s="30">
         <f>IF('DATOS'!$B$35="","-",'DATOS'!$B$35)</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="28" t="n">
+      <c r="A29" s="29" t="n">
         <v>22</v>
       </c>
-      <c r="B29" s="16" t="inlineStr">
+      <c r="B29" s="17" t="inlineStr">
         <is>
           <t>¿Era posible transferir los datos?</t>
         </is>
       </c>
-      <c r="E29" s="29">
+      <c r="E29" s="30">
         <f>IF('DATOS'!$B$36="","-",'DATOS'!$B$36)</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="28" t="n">
+      <c r="A30" s="29" t="n">
         <v>23</v>
       </c>
-      <c r="B30" s="16" t="inlineStr">
+      <c r="B30" s="17" t="inlineStr">
         <is>
           <t>¿Se pudieron descargar todos los datos?</t>
         </is>
       </c>
-      <c r="E30" s="29">
+      <c r="E30" s="30">
         <f>IF('DATOS'!$B$37="","-",'DATOS'!$B$37)</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="28" t="n">
+      <c r="A31" s="29" t="n">
         <v>24</v>
       </c>
-      <c r="B31" s="16" t="inlineStr">
+      <c r="B31" s="17" t="inlineStr">
         <is>
           <t>En caso negativo de 23, ¿por qué?</t>
         </is>
       </c>
-      <c r="E31" s="29">
+      <c r="E31" s="30">
         <f>IF('DATOS'!$B$38="","-",'DATOS'!$B$38)</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="28" t="n">
+      <c r="A32" s="29" t="n">
         <v>25</v>
       </c>
-      <c r="B32" s="16" t="inlineStr">
+      <c r="B32" s="17" t="inlineStr">
         <is>
           <t>Fecha de transferencia de los datos desde la unidad intravehicular</t>
         </is>
       </c>
-      <c r="E32" s="29">
+      <c r="E32" s="30">
         <f>IF('DATOS'!$B$39="","-",IF('DATOS'!$B$39="","",RIGHT("0"&amp;DAY('DATOS'!$B$39),2)&amp;"/"&amp;RIGHT("0"&amp;MONTH('DATOS'!$B$39),2)&amp;"/"&amp;YEAR('DATOS'!$B$39)))</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="28" t="n">
+      <c r="A33" s="29" t="n">
         <v>26</v>
       </c>
-      <c r="B33" s="16" t="inlineStr">
+      <c r="B33" s="17" t="inlineStr">
         <is>
           <t>¿Han sido los datos enviados a la empresa?</t>
         </is>
       </c>
-      <c r="E33" s="29">
+      <c r="E33" s="30">
         <f>IF('DATOS'!$B$40="","-",'DATOS'!$B$40)</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="28" t="n">
+      <c r="A34" s="29" t="n">
         <v>27</v>
       </c>
-      <c r="B34" s="16" t="inlineStr">
+      <c r="B34" s="17" t="inlineStr">
         <is>
           <t>Fecha de envío</t>
         </is>
       </c>
-      <c r="E34" s="29">
+      <c r="E34" s="30">
         <f>IF('DATOS'!$B$41="","-",IF('DATOS'!$B$41="","",RIGHT("0"&amp;DAY('DATOS'!$B$41),2)&amp;"/"&amp;RIGHT("0"&amp;MONTH('DATOS'!$B$41),2)&amp;"/"&amp;YEAR('DATOS'!$B$41)))</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="26" t="inlineStr">
+      <c r="A36" s="27" t="inlineStr">
         <is>
           <t>DECLARACIÓN</t>
         </is>
       </c>
-      <c r="B36" s="27" t="n"/>
-      <c r="C36" s="27" t="n"/>
-      <c r="D36" s="27" t="n"/>
-      <c r="E36" s="27" t="n"/>
-      <c r="F36" s="27" t="n"/>
-      <c r="G36" s="27" t="n"/>
+      <c r="B36" s="28" t="n"/>
+      <c r="C36" s="28" t="n"/>
+      <c r="D36" s="28" t="n"/>
+      <c r="E36" s="28" t="n"/>
+      <c r="F36" s="28" t="n"/>
+      <c r="G36" s="28" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="15" t="inlineStr">
+      <c r="A37" s="16" t="inlineStr">
         <is>
           <t>1  Este documento ha sido emitido de conformidad con los procedimientos establecidos en la Disposición adicional primera del RD 125/2017.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="15">
+      <c r="A38" s="16">
         <f>"2  Este documento atestigua que "&amp;IF('DATOS'!$B$36="Sí","fue posible","no fue posible")&amp;" transferir los datos almacenados en la unidad instalada en el vehículo identificada arriba, con la cual estaba equipado el vehículo identificado arriba. En respuesta a la solicitud por escrito de la empresa de transportes identificada arriba:"</f>
         <v/>
       </c>
     </row>
     <row r="39"/>
     <row r="40">
-      <c r="A40" s="19">
+      <c r="A40" s="20">
         <f>IF('DATOS'!$B$36="Sí","b) Los datos identificados arriba han sido enviados a la empresa de transportes de acuerdo con lo establecido en el Reglamento de ejecución (UE) 2016/799 de la comisión de 18 de marzo de 2016.","a) No han podido serle entregados los datos a la empresa de transportes y este documento se emite como certificado de intransferibilidad de acuerdo con el Reglamento de ejecución (UE) 2016/799 de la comisión de 18 de marzo de 2016.")</f>
         <v/>
       </c>
     </row>
     <row r="41"/>
     <row r="43">
-      <c r="A43" s="21" t="n"/>
-      <c r="E43" s="21" t="n"/>
+      <c r="A43" s="22" t="n"/>
+      <c r="E43" s="22" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="22">
+      <c r="A44" s="23">
         <f>"FIRMA DEL TÉCNICO QUE REALIZÓ LA INTERVENCIÓN: "&amp;IF('DATOS'!$B$29="","-",'DATOS'!$B$29)</f>
         <v/>
       </c>
-      <c r="E44" s="22">
+      <c r="E44" s="23">
         <f>"FIRMA DEL RESPONSABLE TÉCNICO: "&amp;'CONFIGURACION'!$B$15</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="30" t="inlineStr">
+      <c r="A46" s="31" t="inlineStr">
         <is>
           <t>La solicitud por escrito de remisión de los datos transferidos por la empresa de transportes debe ser adjuntada a la copia de este documento que se archive en el centro técnico.</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="23">
+      <c r="A48" s="24">
         <f>"Formato "&amp;'CONFIGURACION'!$B$23&amp;" · Versión "&amp;'CONFIGURACION'!$B$20&amp;" · Edición "&amp;IF('CONFIGURACION'!$B$21="","",RIGHT("0"&amp;DAY('CONFIGURACION'!$B$21),2)&amp;"/"&amp;RIGHT("0"&amp;MONTH('CONFIGURACION'!$B$21),2)&amp;"/"&amp;YEAR('CONFIGURACION'!$B$21))&amp;" · Elaborado: "&amp;'CONFIGURACION'!$B$16&amp;" · Aprobado: "&amp;'CONFIGURACION'!$B$17&amp;" · UNE 66102:2025"</f>
         <v/>
       </c>
@@ -2505,63 +2510,63 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12">
+      <c r="A1" s="13">
         <f>'CONFIGURACION'!$B$4</f>
         <v/>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="14">
+      <c r="A2" s="15">
         <f>'CONFIGURACION'!$B$5</f>
         <v/>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14">
+      <c r="A3" s="15">
         <f>'CONFIGURACION'!$B$6</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="14">
+      <c r="A4" s="15">
         <f>'CONFIGURACION'!$B$7</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="14">
+      <c r="A5" s="15">
         <f>'CONFIGURACION'!$B$8</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="14">
+      <c r="A6" s="15">
         <f>'CONFIGURACION'!$B$9</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="31" t="inlineStr">
+      <c r="A9" s="32" t="inlineStr">
         <is>
           <t>Acuse de recibo Certificado de Intransferibilidad de datos</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12">
+      <c r="A11" s="13">
         <f>IF('DATOS'!$B$5="","",'DATOS'!$B$5)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="14" t="inlineStr">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>Estimados señores:</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="15" t="inlineStr">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>En cumplimiento del requisito expresado en la disposición adicional primera, apartado 10, del Real decreto 125:2017, les remitimos copia del certificado de intransferibilidad correspondiente a la sustitución del tacógrafo:</t>
         </is>
@@ -2570,84 +2575,84 @@
     <row r="17"/>
     <row r="18"/>
     <row r="20">
-      <c r="A20" s="14" t="inlineStr">
+      <c r="A20" s="15" t="inlineStr">
         <is>
           <t>Modelo:</t>
         </is>
       </c>
-      <c r="C20" s="12">
+      <c r="C20" s="13">
         <f>IF('DATOS'!$B$18="","",'DATOS'!$B$18)</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="14" t="inlineStr">
+      <c r="A21" s="15" t="inlineStr">
         <is>
           <t>Nº de Serie:</t>
         </is>
       </c>
-      <c r="C21" s="12">
+      <c r="C21" s="13">
         <f>IF('DATOS'!$B$19="","",'DATOS'!$B$19)</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="14" t="inlineStr">
+      <c r="A23" s="15" t="inlineStr">
         <is>
           <t>Montado en el vehículo:</t>
         </is>
       </c>
-      <c r="C23" s="12">
+      <c r="C23" s="13">
         <f>UPPER(IF('DATOS'!$B$12="","",'DATOS'!$B$12))</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="14" t="inlineStr">
+      <c r="A24" s="15" t="inlineStr">
         <is>
           <t>Nº de informe/Certificado:</t>
         </is>
       </c>
-      <c r="C24" s="12">
+      <c r="C24" s="13">
         <f>IF('DATOS'!$B$25="","",'DATOS'!$B$25)</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="14" t="inlineStr">
+      <c r="A25" s="15" t="inlineStr">
         <is>
           <t>Fecha Informe:</t>
         </is>
       </c>
-      <c r="C25" s="32">
+      <c r="C25" s="33">
         <f>IF('DATOS'!$B$26="","",'DATOS'!$B$26)</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="14" t="inlineStr">
+      <c r="A27" s="15" t="inlineStr">
         <is>
           <t>Nombre:</t>
         </is>
       </c>
-      <c r="C27" s="12">
+      <c r="C27" s="13">
         <f>IF('DATOS'!$B$8="","",'DATOS'!$B$8)</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="14" t="inlineStr">
+      <c r="A28" s="15" t="inlineStr">
         <is>
           <t>DNI:</t>
         </is>
       </c>
-      <c r="C28" s="12">
+      <c r="C28" s="13">
         <f>IF('DATOS'!$B$9="","",'DATOS'!$B$9)</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="15">
+      <c r="A30" s="16">
         <f>"En calidad de personal/propietario de la organización de transportes propietaria del vehículo con matrícula "&amp;UPPER(IF('DATOS'!$B$12="","",'DATOS'!$B$12))&amp;" declaro haber recibido el certificado de intransferibilidad de fecha "&amp;IF('DATOS'!$B$26="","",RIGHT("0"&amp;DAY('DATOS'!$B$26),2)&amp;"/"&amp;RIGHT("0"&amp;MONTH('DATOS'!$B$26),2)&amp;"/"&amp;YEAR('DATOS'!$B$26))&amp;" correspondiente a la intervención técnica realizada sobre el vehículo de matrícula antedicha."</f>
         <v/>
       </c>
@@ -2655,7 +2660,7 @@
     <row r="31"/>
     <row r="32"/>
     <row r="34">
-      <c r="A34" s="15" t="inlineStr">
+      <c r="A34" s="16" t="inlineStr">
         <is>
           <t>En el caso de que el receptor no sea propietario de la organización de transportes, se compromete explícitamente, por el presente compromiso firmado, a entregar este documento (el certificado de intransferibilidad) a la propiedad de la citada organización</t>
         </is>
@@ -2664,59 +2669,59 @@
     <row r="35"/>
     <row r="36"/>
     <row r="38">
-      <c r="A38" s="12">
+      <c r="A38" s="13">
         <f>IF('DATOS'!$B$45="Sí",'CONFIGURACION'!$B$50,"")</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="12">
+      <c r="A39" s="13">
         <f>IF('DATOS'!$B$46="Sí",'CONFIGURACION'!$B$51,"")</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="18">
+      <c r="A41" s="19">
         <f>'CONFIGURACION'!$B$53</f>
         <v/>
       </c>
     </row>
     <row r="42"/>
     <row r="44">
-      <c r="A44" s="14" t="inlineStr">
+      <c r="A44" s="15" t="inlineStr">
         <is>
           <t>Entregado</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="14">
+      <c r="A45" s="15">
         <f>'CONFIGURACION'!$B$10&amp;" a"</f>
         <v/>
       </c>
-      <c r="C45" s="32">
+      <c r="C45" s="33">
         <f>IF('DATOS'!$B$27="","",'DATOS'!$B$27)</f>
         <v/>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="14" t="inlineStr">
+      <c r="A47" s="15" t="inlineStr">
         <is>
           <t>Firma:</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="B48" s="21" t="n"/>
+      <c r="B48" s="22" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="20">
+      <c r="A50" s="21">
         <f>IF('DATOS'!$B$28="Intransferibilidad","","— NO APLICA: esta intervención está marcada como Transferencia correcta —")</f>
         <v/>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="23">
+      <c r="A52" s="24">
         <f>"Formato "&amp;'CONFIGURACION'!$B$24&amp;" · Versión "&amp;'CONFIGURACION'!$B$20&amp;" · Edición "&amp;IF('CONFIGURACION'!$B$21="","",RIGHT("0"&amp;DAY('CONFIGURACION'!$B$21),2)&amp;"/"&amp;RIGHT("0"&amp;MONTH('CONFIGURACION'!$B$21),2)&amp;"/"&amp;YEAR('CONFIGURACION'!$B$21))&amp;" · Elaborado: "&amp;'CONFIGURACION'!$B$16&amp;" · Aprobado: "&amp;'CONFIGURACION'!$B$17&amp;" · UNE 66102:2025"</f>
         <v/>
       </c>
@@ -2774,63 +2779,63 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12">
+      <c r="A1" s="13">
         <f>'CONFIGURACION'!$B$4</f>
         <v/>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="14">
+      <c r="A2" s="15">
         <f>'CONFIGURACION'!$B$5</f>
         <v/>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14">
+      <c r="A3" s="15">
         <f>'CONFIGURACION'!$B$6</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="14">
+      <c r="A4" s="15">
         <f>'CONFIGURACION'!$B$7</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="14">
+      <c r="A5" s="15">
         <f>'CONFIGURACION'!$B$8</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="14">
+      <c r="A6" s="15">
         <f>'CONFIGURACION'!$B$9</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="31" t="inlineStr">
+      <c r="A9" s="32" t="inlineStr">
         <is>
           <t>Acuse de recibo Certificado de Intransferibilidad de datos</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12">
+      <c r="A11" s="13">
         <f>'CONFIGURACION'!$B$12</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="14" t="inlineStr">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>Estimados señores:</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="15" t="inlineStr">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>En cumplimiento del requisito expresado en la disposición adicional primera, apartado 10, del Real decreto 125:2017, les remitimos copia del certificado de intransferibilidad correspondiente a la sustitución del tacógrafo:</t>
         </is>
@@ -2839,85 +2844,85 @@
     <row r="17"/>
     <row r="18"/>
     <row r="20">
-      <c r="A20" s="14" t="inlineStr">
+      <c r="A20" s="15" t="inlineStr">
         <is>
           <t>Modelo:</t>
         </is>
       </c>
-      <c r="C20" s="12">
+      <c r="C20" s="13">
         <f>IF('DATOS'!$B$18="","",'DATOS'!$B$18)</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="14" t="inlineStr">
+      <c r="A21" s="15" t="inlineStr">
         <is>
           <t>Nº de Serie:</t>
         </is>
       </c>
-      <c r="C21" s="12">
+      <c r="C21" s="13">
         <f>IF('DATOS'!$B$19="","",'DATOS'!$B$19)</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="14" t="inlineStr">
+      <c r="A23" s="15" t="inlineStr">
         <is>
           <t>Montado en el vehículo:</t>
         </is>
       </c>
-      <c r="C23" s="12">
+      <c r="C23" s="13">
         <f>UPPER(IF('DATOS'!$B$12="","",'DATOS'!$B$12))</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="14" t="inlineStr">
+      <c r="A24" s="15" t="inlineStr">
         <is>
           <t>Nº de informe/Certificado:</t>
         </is>
       </c>
-      <c r="C24" s="12">
+      <c r="C24" s="13">
         <f>IF('DATOS'!$B$25="","",'DATOS'!$B$25)</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="14" t="inlineStr">
+      <c r="A25" s="15" t="inlineStr">
         <is>
           <t>Fecha Informe:</t>
         </is>
       </c>
-      <c r="C25" s="32">
+      <c r="C25" s="33">
         <f>IF('DATOS'!$B$26="","",'DATOS'!$B$26)</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="14" t="inlineStr">
+      <c r="A28" s="15" t="inlineStr">
         <is>
           <t>Entregado</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="14">
+      <c r="A29" s="15">
         <f>'CONFIGURACION'!$B$10&amp;" a"</f>
         <v/>
       </c>
-      <c r="C29" s="32">
+      <c r="C29" s="33">
         <f>IF('DATOS'!$B$27="","",'DATOS'!$B$27)</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="20">
+      <c r="A32" s="21">
         <f>IF('DATOS'!$B$28="Intransferibilidad","","— NO APLICA: esta intervención está marcada como Transferencia correcta —")</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="23">
+      <c r="A34" s="24">
         <f>"Formato "&amp;'CONFIGURACION'!$B$25&amp;" · Versión "&amp;'CONFIGURACION'!$B$20&amp;" · Edición "&amp;IF('CONFIGURACION'!$B$21="","",RIGHT("0"&amp;DAY('CONFIGURACION'!$B$21),2)&amp;"/"&amp;RIGHT("0"&amp;MONTH('CONFIGURACION'!$B$21),2)&amp;"/"&amp;YEAR('CONFIGURACION'!$B$21))&amp;" · Elaborado: "&amp;'CONFIGURACION'!$B$16&amp;" · Aprobado: "&amp;'CONFIGURACION'!$B$17&amp;" · UNE 66102:2025"</f>
         <v/>
       </c>
@@ -2973,7 +2978,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="33">
+      <c r="A45" s="34">
         <f>'CONFIGURACION'!$B$56&amp;IF('DATOS'!$B$18="","",'DATOS'!$B$18)&amp;'CONFIGURACION'!$B$57&amp;IF('DATOS'!$B$19="","",'DATOS'!$B$19)&amp;'CONFIGURACION'!$B$58&amp;UPPER(IF('DATOS'!$B$12="","",'DATOS'!$B$12))&amp;'CONFIGURACION'!$B$59&amp;IF('DATOS'!$B$25="","",'DATOS'!$B$25)&amp;'CONFIGURACION'!$B$60&amp;IF('DATOS'!$B$26="","",RIGHT("0"&amp;DAY('DATOS'!$B$26),2)&amp;"/"&amp;RIGHT("0"&amp;MONTH('DATOS'!$B$26),2)&amp;"/"&amp;YEAR('DATOS'!$B$26))&amp;'CONFIGURACION'!$B$61</f>
         <v/>
       </c>
@@ -2988,7 +2993,7 @@
           <t>Enlace al trámite:</t>
         </is>
       </c>
-      <c r="C51" s="34">
+      <c r="C51" s="35">
         <f>HYPERLINK('CONFIGURACION'!$B$30,"Petició genèrica — gencat.cat")</f>
         <v/>
       </c>
@@ -2999,7 +3004,7 @@
           <t>Formulario directo (OVT):</t>
         </is>
       </c>
-      <c r="C52" s="34">
+      <c r="C52" s="35">
         <f>HYPERLINK('CONFIGURACION'!$B$31,"Obrir el formulari a l’OVT")</f>
         <v/>
       </c>
@@ -3081,134 +3086,134 @@
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="35" t="inlineStr">
+      <c r="A2" s="36" t="inlineStr">
         <is>
           <t>UNE 66102:2025, 7.5.1 d) y 8.5.1 — registro de transferencias realizadas y documento de destrucción al año. La fila 5 se rellena sola con la intervención en curso; cópiala como valores a la primera fila libre al cerrar cada expediente.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="34" customHeight="1">
-      <c r="A4" s="36" t="inlineStr">
+      <c r="A4" s="37" t="inlineStr">
         <is>
           <t>Nº informe</t>
         </is>
       </c>
-      <c r="B4" s="36" t="inlineStr">
+      <c r="B4" s="37" t="inlineStr">
         <is>
           <t>Fecha transferencia</t>
         </is>
       </c>
-      <c r="C4" s="36" t="inlineStr">
+      <c r="C4" s="37" t="inlineStr">
         <is>
           <t>Matrícula</t>
         </is>
       </c>
-      <c r="D4" s="36" t="inlineStr">
+      <c r="D4" s="37" t="inlineStr">
         <is>
           <t>Nº bastidor</t>
         </is>
       </c>
-      <c r="E4" s="36" t="inlineStr">
+      <c r="E4" s="37" t="inlineStr">
         <is>
           <t>Nº serie UIV</t>
         </is>
       </c>
-      <c r="F4" s="36" t="inlineStr">
+      <c r="F4" s="37" t="inlineStr">
         <is>
           <t>Empresa</t>
         </is>
       </c>
-      <c r="G4" s="36" t="inlineStr">
+      <c r="G4" s="37" t="inlineStr">
         <is>
           <t>Técnico</t>
         </is>
       </c>
-      <c r="H4" s="36" t="inlineStr">
+      <c r="H4" s="37" t="inlineStr">
         <is>
           <t>Modalidad entrega</t>
         </is>
       </c>
-      <c r="I4" s="36" t="inlineStr">
+      <c r="I4" s="37" t="inlineStr">
         <is>
           <t>Fecha envío</t>
         </is>
       </c>
-      <c r="J4" s="36" t="inlineStr">
+      <c r="J4" s="37" t="inlineStr">
         <is>
           <t>Destruir a partir de</t>
         </is>
       </c>
-      <c r="K4" s="36" t="inlineStr">
+      <c r="K4" s="37" t="inlineStr">
         <is>
           <t>Fecha destrucción</t>
         </is>
       </c>
-      <c r="L4" s="36" t="inlineStr">
+      <c r="L4" s="37" t="inlineStr">
         <is>
           <t>Método de destrucción</t>
         </is>
       </c>
-      <c r="M4" s="36" t="inlineStr">
+      <c r="M4" s="37" t="inlineStr">
         <is>
           <t>Persona que destruye</t>
         </is>
       </c>
-      <c r="N4" s="36" t="inlineStr">
+      <c r="N4" s="37" t="inlineStr">
         <is>
           <t>Firma digital del archivo (hash)</t>
         </is>
       </c>
-      <c r="O4" s="36" t="inlineStr">
+      <c r="O4" s="37" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="37">
+      <c r="A5" s="38">
         <f>IF('DATOS'!$B$25="","",'DATOS'!$B$25)</f>
         <v/>
       </c>
-      <c r="B5" s="38">
+      <c r="B5" s="39">
         <f>IF('DATOS'!$B$39="","",'DATOS'!$B$39)</f>
         <v/>
       </c>
-      <c r="C5" s="37">
+      <c r="C5" s="38">
         <f>UPPER(IF('DATOS'!$B$12="","",'DATOS'!$B$12))</f>
         <v/>
       </c>
-      <c r="D5" s="37">
+      <c r="D5" s="38">
         <f>IF('DATOS'!$B$13="","",'DATOS'!$B$13)</f>
         <v/>
       </c>
-      <c r="E5" s="37">
+      <c r="E5" s="38">
         <f>IF('DATOS'!$B$19="","",'DATOS'!$B$19)</f>
         <v/>
       </c>
-      <c r="F5" s="37">
+      <c r="F5" s="38">
         <f>IF('DATOS'!$B$5="","",'DATOS'!$B$5)</f>
         <v/>
       </c>
-      <c r="G5" s="37">
+      <c r="G5" s="38">
         <f>IF('DATOS'!$B$29="","",'DATOS'!$B$29)</f>
         <v/>
       </c>
-      <c r="H5" s="37">
+      <c r="H5" s="38">
         <f>IF('DATOS'!$B$43="","",'DATOS'!$B$43)</f>
         <v/>
       </c>
-      <c r="I5" s="38">
+      <c r="I5" s="39">
         <f>IF('DATOS'!$B$41="","",'DATOS'!$B$41)</f>
         <v/>
       </c>
-      <c r="J5" s="38">
+      <c r="J5" s="39">
         <f>IF('DATOS'!$B$39="","",EDATE('DATOS'!$B$39,12))</f>
         <v/>
       </c>
-      <c r="K5" s="39" t="n"/>
-      <c r="L5" s="39" t="n"/>
-      <c r="M5" s="39" t="n"/>
-      <c r="N5" s="39" t="n"/>
+      <c r="K5" s="40" t="n"/>
+      <c r="L5" s="40" t="n"/>
+      <c r="M5" s="40" t="n"/>
+      <c r="N5" s="40" t="n"/>
       <c r="O5" s="2" t="inlineStr">
         <is>
           <t>← intervención en curso (automática)</t>
@@ -3216,783 +3221,783 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="40" t="n"/>
-      <c r="B6" s="41" t="n"/>
-      <c r="C6" s="40" t="n"/>
-      <c r="D6" s="40" t="n"/>
-      <c r="E6" s="40" t="n"/>
-      <c r="F6" s="40" t="n"/>
-      <c r="G6" s="40" t="n"/>
-      <c r="H6" s="40" t="n"/>
-      <c r="I6" s="41" t="n"/>
-      <c r="J6" s="42">
+      <c r="A6" s="41" t="n"/>
+      <c r="B6" s="42" t="n"/>
+      <c r="C6" s="41" t="n"/>
+      <c r="D6" s="41" t="n"/>
+      <c r="E6" s="41" t="n"/>
+      <c r="F6" s="41" t="n"/>
+      <c r="G6" s="41" t="n"/>
+      <c r="H6" s="41" t="n"/>
+      <c r="I6" s="42" t="n"/>
+      <c r="J6" s="43">
         <f>IF(B6="","",EDATE(B6,12))</f>
         <v/>
       </c>
-      <c r="K6" s="41" t="n"/>
-      <c r="L6" s="40" t="n"/>
-      <c r="M6" s="40" t="n"/>
-      <c r="N6" s="40" t="n"/>
-      <c r="O6" s="43">
+      <c r="K6" s="42" t="n"/>
+      <c r="L6" s="41" t="n"/>
+      <c r="M6" s="41" t="n"/>
+      <c r="N6" s="41" t="n"/>
+      <c r="O6" s="44">
         <f>IF(B6="","",IF(K6&lt;&gt;"","Destruido",IF(TODAY()&gt;EDATE(B6,12),"⚠ PENDIENTE DE DESTRUIR","En custodia")))</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="40" t="n"/>
-      <c r="B7" s="41" t="n"/>
-      <c r="C7" s="40" t="n"/>
-      <c r="D7" s="40" t="n"/>
-      <c r="E7" s="40" t="n"/>
-      <c r="F7" s="40" t="n"/>
-      <c r="G7" s="40" t="n"/>
-      <c r="H7" s="40" t="n"/>
-      <c r="I7" s="41" t="n"/>
-      <c r="J7" s="42">
+      <c r="A7" s="41" t="n"/>
+      <c r="B7" s="42" t="n"/>
+      <c r="C7" s="41" t="n"/>
+      <c r="D7" s="41" t="n"/>
+      <c r="E7" s="41" t="n"/>
+      <c r="F7" s="41" t="n"/>
+      <c r="G7" s="41" t="n"/>
+      <c r="H7" s="41" t="n"/>
+      <c r="I7" s="42" t="n"/>
+      <c r="J7" s="43">
         <f>IF(B7="","",EDATE(B7,12))</f>
         <v/>
       </c>
-      <c r="K7" s="41" t="n"/>
-      <c r="L7" s="40" t="n"/>
-      <c r="M7" s="40" t="n"/>
-      <c r="N7" s="40" t="n"/>
-      <c r="O7" s="43">
+      <c r="K7" s="42" t="n"/>
+      <c r="L7" s="41" t="n"/>
+      <c r="M7" s="41" t="n"/>
+      <c r="N7" s="41" t="n"/>
+      <c r="O7" s="44">
         <f>IF(B7="","",IF(K7&lt;&gt;"","Destruido",IF(TODAY()&gt;EDATE(B7,12),"⚠ PENDIENTE DE DESTRUIR","En custodia")))</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="40" t="n"/>
-      <c r="B8" s="41" t="n"/>
-      <c r="C8" s="40" t="n"/>
-      <c r="D8" s="40" t="n"/>
-      <c r="E8" s="40" t="n"/>
-      <c r="F8" s="40" t="n"/>
-      <c r="G8" s="40" t="n"/>
-      <c r="H8" s="40" t="n"/>
-      <c r="I8" s="41" t="n"/>
-      <c r="J8" s="42">
+      <c r="A8" s="41" t="n"/>
+      <c r="B8" s="42" t="n"/>
+      <c r="C8" s="41" t="n"/>
+      <c r="D8" s="41" t="n"/>
+      <c r="E8" s="41" t="n"/>
+      <c r="F8" s="41" t="n"/>
+      <c r="G8" s="41" t="n"/>
+      <c r="H8" s="41" t="n"/>
+      <c r="I8" s="42" t="n"/>
+      <c r="J8" s="43">
         <f>IF(B8="","",EDATE(B8,12))</f>
         <v/>
       </c>
-      <c r="K8" s="41" t="n"/>
-      <c r="L8" s="40" t="n"/>
-      <c r="M8" s="40" t="n"/>
-      <c r="N8" s="40" t="n"/>
-      <c r="O8" s="43">
+      <c r="K8" s="42" t="n"/>
+      <c r="L8" s="41" t="n"/>
+      <c r="M8" s="41" t="n"/>
+      <c r="N8" s="41" t="n"/>
+      <c r="O8" s="44">
         <f>IF(B8="","",IF(K8&lt;&gt;"","Destruido",IF(TODAY()&gt;EDATE(B8,12),"⚠ PENDIENTE DE DESTRUIR","En custodia")))</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="40" t="n"/>
-      <c r="B9" s="41" t="n"/>
-      <c r="C9" s="40" t="n"/>
-      <c r="D9" s="40" t="n"/>
-      <c r="E9" s="40" t="n"/>
-      <c r="F9" s="40" t="n"/>
-      <c r="G9" s="40" t="n"/>
-      <c r="H9" s="40" t="n"/>
-      <c r="I9" s="41" t="n"/>
-      <c r="J9" s="42">
+      <c r="A9" s="41" t="n"/>
+      <c r="B9" s="42" t="n"/>
+      <c r="C9" s="41" t="n"/>
+      <c r="D9" s="41" t="n"/>
+      <c r="E9" s="41" t="n"/>
+      <c r="F9" s="41" t="n"/>
+      <c r="G9" s="41" t="n"/>
+      <c r="H9" s="41" t="n"/>
+      <c r="I9" s="42" t="n"/>
+      <c r="J9" s="43">
         <f>IF(B9="","",EDATE(B9,12))</f>
         <v/>
       </c>
-      <c r="K9" s="41" t="n"/>
-      <c r="L9" s="40" t="n"/>
-      <c r="M9" s="40" t="n"/>
-      <c r="N9" s="40" t="n"/>
-      <c r="O9" s="43">
+      <c r="K9" s="42" t="n"/>
+      <c r="L9" s="41" t="n"/>
+      <c r="M9" s="41" t="n"/>
+      <c r="N9" s="41" t="n"/>
+      <c r="O9" s="44">
         <f>IF(B9="","",IF(K9&lt;&gt;"","Destruido",IF(TODAY()&gt;EDATE(B9,12),"⚠ PENDIENTE DE DESTRUIR","En custodia")))</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="40" t="n"/>
-      <c r="B10" s="41" t="n"/>
-      <c r="C10" s="40" t="n"/>
-      <c r="D10" s="40" t="n"/>
-      <c r="E10" s="40" t="n"/>
-      <c r="F10" s="40" t="n"/>
-      <c r="G10" s="40" t="n"/>
-      <c r="H10" s="40" t="n"/>
-      <c r="I10" s="41" t="n"/>
-      <c r="J10" s="42">
+      <c r="A10" s="41" t="n"/>
+      <c r="B10" s="42" t="n"/>
+      <c r="C10" s="41" t="n"/>
+      <c r="D10" s="41" t="n"/>
+      <c r="E10" s="41" t="n"/>
+      <c r="F10" s="41" t="n"/>
+      <c r="G10" s="41" t="n"/>
+      <c r="H10" s="41" t="n"/>
+      <c r="I10" s="42" t="n"/>
+      <c r="J10" s="43">
         <f>IF(B10="","",EDATE(B10,12))</f>
         <v/>
       </c>
-      <c r="K10" s="41" t="n"/>
-      <c r="L10" s="40" t="n"/>
-      <c r="M10" s="40" t="n"/>
-      <c r="N10" s="40" t="n"/>
-      <c r="O10" s="43">
+      <c r="K10" s="42" t="n"/>
+      <c r="L10" s="41" t="n"/>
+      <c r="M10" s="41" t="n"/>
+      <c r="N10" s="41" t="n"/>
+      <c r="O10" s="44">
         <f>IF(B10="","",IF(K10&lt;&gt;"","Destruido",IF(TODAY()&gt;EDATE(B10,12),"⚠ PENDIENTE DE DESTRUIR","En custodia")))</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="40" t="n"/>
-      <c r="B11" s="41" t="n"/>
-      <c r="C11" s="40" t="n"/>
-      <c r="D11" s="40" t="n"/>
-      <c r="E11" s="40" t="n"/>
-      <c r="F11" s="40" t="n"/>
-      <c r="G11" s="40" t="n"/>
-      <c r="H11" s="40" t="n"/>
-      <c r="I11" s="41" t="n"/>
-      <c r="J11" s="42">
+      <c r="A11" s="41" t="n"/>
+      <c r="B11" s="42" t="n"/>
+      <c r="C11" s="41" t="n"/>
+      <c r="D11" s="41" t="n"/>
+      <c r="E11" s="41" t="n"/>
+      <c r="F11" s="41" t="n"/>
+      <c r="G11" s="41" t="n"/>
+      <c r="H11" s="41" t="n"/>
+      <c r="I11" s="42" t="n"/>
+      <c r="J11" s="43">
         <f>IF(B11="","",EDATE(B11,12))</f>
         <v/>
       </c>
-      <c r="K11" s="41" t="n"/>
-      <c r="L11" s="40" t="n"/>
-      <c r="M11" s="40" t="n"/>
-      <c r="N11" s="40" t="n"/>
-      <c r="O11" s="43">
+      <c r="K11" s="42" t="n"/>
+      <c r="L11" s="41" t="n"/>
+      <c r="M11" s="41" t="n"/>
+      <c r="N11" s="41" t="n"/>
+      <c r="O11" s="44">
         <f>IF(B11="","",IF(K11&lt;&gt;"","Destruido",IF(TODAY()&gt;EDATE(B11,12),"⚠ PENDIENTE DE DESTRUIR","En custodia")))</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="40" t="n"/>
-      <c r="B12" s="41" t="n"/>
-      <c r="C12" s="40" t="n"/>
-      <c r="D12" s="40" t="n"/>
-      <c r="E12" s="40" t="n"/>
-      <c r="F12" s="40" t="n"/>
-      <c r="G12" s="40" t="n"/>
-      <c r="H12" s="40" t="n"/>
-      <c r="I12" s="41" t="n"/>
-      <c r="J12" s="42">
+      <c r="A12" s="41" t="n"/>
+      <c r="B12" s="42" t="n"/>
+      <c r="C12" s="41" t="n"/>
+      <c r="D12" s="41" t="n"/>
+      <c r="E12" s="41" t="n"/>
+      <c r="F12" s="41" t="n"/>
+      <c r="G12" s="41" t="n"/>
+      <c r="H12" s="41" t="n"/>
+      <c r="I12" s="42" t="n"/>
+      <c r="J12" s="43">
         <f>IF(B12="","",EDATE(B12,12))</f>
         <v/>
       </c>
-      <c r="K12" s="41" t="n"/>
-      <c r="L12" s="40" t="n"/>
-      <c r="M12" s="40" t="n"/>
-      <c r="N12" s="40" t="n"/>
-      <c r="O12" s="43">
+      <c r="K12" s="42" t="n"/>
+      <c r="L12" s="41" t="n"/>
+      <c r="M12" s="41" t="n"/>
+      <c r="N12" s="41" t="n"/>
+      <c r="O12" s="44">
         <f>IF(B12="","",IF(K12&lt;&gt;"","Destruido",IF(TODAY()&gt;EDATE(B12,12),"⚠ PENDIENTE DE DESTRUIR","En custodia")))</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="40" t="n"/>
-      <c r="B13" s="41" t="n"/>
-      <c r="C13" s="40" t="n"/>
-      <c r="D13" s="40" t="n"/>
-      <c r="E13" s="40" t="n"/>
-      <c r="F13" s="40" t="n"/>
-      <c r="G13" s="40" t="n"/>
-      <c r="H13" s="40" t="n"/>
-      <c r="I13" s="41" t="n"/>
-      <c r="J13" s="42">
+      <c r="A13" s="41" t="n"/>
+      <c r="B13" s="42" t="n"/>
+      <c r="C13" s="41" t="n"/>
+      <c r="D13" s="41" t="n"/>
+      <c r="E13" s="41" t="n"/>
+      <c r="F13" s="41" t="n"/>
+      <c r="G13" s="41" t="n"/>
+      <c r="H13" s="41" t="n"/>
+      <c r="I13" s="42" t="n"/>
+      <c r="J13" s="43">
         <f>IF(B13="","",EDATE(B13,12))</f>
         <v/>
       </c>
-      <c r="K13" s="41" t="n"/>
-      <c r="L13" s="40" t="n"/>
-      <c r="M13" s="40" t="n"/>
-      <c r="N13" s="40" t="n"/>
-      <c r="O13" s="43">
+      <c r="K13" s="42" t="n"/>
+      <c r="L13" s="41" t="n"/>
+      <c r="M13" s="41" t="n"/>
+      <c r="N13" s="41" t="n"/>
+      <c r="O13" s="44">
         <f>IF(B13="","",IF(K13&lt;&gt;"","Destruido",IF(TODAY()&gt;EDATE(B13,12),"⚠ PENDIENTE DE DESTRUIR","En custodia")))</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="40" t="n"/>
-      <c r="B14" s="41" t="n"/>
-      <c r="C14" s="40" t="n"/>
-      <c r="D14" s="40" t="n"/>
-      <c r="E14" s="40" t="n"/>
-      <c r="F14" s="40" t="n"/>
-      <c r="G14" s="40" t="n"/>
-      <c r="H14" s="40" t="n"/>
-      <c r="I14" s="41" t="n"/>
-      <c r="J14" s="42">
+      <c r="A14" s="41" t="n"/>
+      <c r="B14" s="42" t="n"/>
+      <c r="C14" s="41" t="n"/>
+      <c r="D14" s="41" t="n"/>
+      <c r="E14" s="41" t="n"/>
+      <c r="F14" s="41" t="n"/>
+      <c r="G14" s="41" t="n"/>
+      <c r="H14" s="41" t="n"/>
+      <c r="I14" s="42" t="n"/>
+      <c r="J14" s="43">
         <f>IF(B14="","",EDATE(B14,12))</f>
         <v/>
       </c>
-      <c r="K14" s="41" t="n"/>
-      <c r="L14" s="40" t="n"/>
-      <c r="M14" s="40" t="n"/>
-      <c r="N14" s="40" t="n"/>
-      <c r="O14" s="43">
+      <c r="K14" s="42" t="n"/>
+      <c r="L14" s="41" t="n"/>
+      <c r="M14" s="41" t="n"/>
+      <c r="N14" s="41" t="n"/>
+      <c r="O14" s="44">
         <f>IF(B14="","",IF(K14&lt;&gt;"","Destruido",IF(TODAY()&gt;EDATE(B14,12),"⚠ PENDIENTE DE DESTRUIR","En custodia")))</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="40" t="n"/>
-      <c r="B15" s="41" t="n"/>
-      <c r="C15" s="40" t="n"/>
-      <c r="D15" s="40" t="n"/>
-      <c r="E15" s="40" t="n"/>
-      <c r="F15" s="40" t="n"/>
-      <c r="G15" s="40" t="n"/>
-      <c r="H15" s="40" t="n"/>
-      <c r="I15" s="41" t="n"/>
-      <c r="J15" s="42">
+      <c r="A15" s="41" t="n"/>
+      <c r="B15" s="42" t="n"/>
+      <c r="C15" s="41" t="n"/>
+      <c r="D15" s="41" t="n"/>
+      <c r="E15" s="41" t="n"/>
+      <c r="F15" s="41" t="n"/>
+      <c r="G15" s="41" t="n"/>
+      <c r="H15" s="41" t="n"/>
+      <c r="I15" s="42" t="n"/>
+      <c r="J15" s="43">
         <f>IF(B15="","",EDATE(B15,12))</f>
         <v/>
       </c>
-      <c r="K15" s="41" t="n"/>
-      <c r="L15" s="40" t="n"/>
-      <c r="M15" s="40" t="n"/>
-      <c r="N15" s="40" t="n"/>
-      <c r="O15" s="43">
+      <c r="K15" s="42" t="n"/>
+      <c r="L15" s="41" t="n"/>
+      <c r="M15" s="41" t="n"/>
+      <c r="N15" s="41" t="n"/>
+      <c r="O15" s="44">
         <f>IF(B15="","",IF(K15&lt;&gt;"","Destruido",IF(TODAY()&gt;EDATE(B15,12),"⚠ PENDIENTE DE DESTRUIR","En custodia")))</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="40" t="n"/>
-      <c r="B16" s="41" t="n"/>
-      <c r="C16" s="40" t="n"/>
-      <c r="D16" s="40" t="n"/>
-      <c r="E16" s="40" t="n"/>
-      <c r="F16" s="40" t="n"/>
-      <c r="G16" s="40" t="n"/>
-      <c r="H16" s="40" t="n"/>
-      <c r="I16" s="41" t="n"/>
-      <c r="J16" s="42">
+      <c r="A16" s="41" t="n"/>
+      <c r="B16" s="42" t="n"/>
+      <c r="C16" s="41" t="n"/>
+      <c r="D16" s="41" t="n"/>
+      <c r="E16" s="41" t="n"/>
+      <c r="F16" s="41" t="n"/>
+      <c r="G16" s="41" t="n"/>
+      <c r="H16" s="41" t="n"/>
+      <c r="I16" s="42" t="n"/>
+      <c r="J16" s="43">
         <f>IF(B16="","",EDATE(B16,12))</f>
         <v/>
       </c>
-      <c r="K16" s="41" t="n"/>
-      <c r="L16" s="40" t="n"/>
-      <c r="M16" s="40" t="n"/>
-      <c r="N16" s="40" t="n"/>
-      <c r="O16" s="43">
+      <c r="K16" s="42" t="n"/>
+      <c r="L16" s="41" t="n"/>
+      <c r="M16" s="41" t="n"/>
+      <c r="N16" s="41" t="n"/>
+      <c r="O16" s="44">
         <f>IF(B16="","",IF(K16&lt;&gt;"","Destruido",IF(TODAY()&gt;EDATE(B16,12),"⚠ PENDIENTE DE DESTRUIR","En custodia")))</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="40" t="n"/>
-      <c r="B17" s="41" t="n"/>
-      <c r="C17" s="40" t="n"/>
-      <c r="D17" s="40" t="n"/>
-      <c r="E17" s="40" t="n"/>
-      <c r="F17" s="40" t="n"/>
-      <c r="G17" s="40" t="n"/>
-      <c r="H17" s="40" t="n"/>
-      <c r="I17" s="41" t="n"/>
-      <c r="J17" s="42">
+      <c r="A17" s="41" t="n"/>
+      <c r="B17" s="42" t="n"/>
+      <c r="C17" s="41" t="n"/>
+      <c r="D17" s="41" t="n"/>
+      <c r="E17" s="41" t="n"/>
+      <c r="F17" s="41" t="n"/>
+      <c r="G17" s="41" t="n"/>
+      <c r="H17" s="41" t="n"/>
+      <c r="I17" s="42" t="n"/>
+      <c r="J17" s="43">
         <f>IF(B17="","",EDATE(B17,12))</f>
         <v/>
       </c>
-      <c r="K17" s="41" t="n"/>
-      <c r="L17" s="40" t="n"/>
-      <c r="M17" s="40" t="n"/>
-      <c r="N17" s="40" t="n"/>
-      <c r="O17" s="43">
+      <c r="K17" s="42" t="n"/>
+      <c r="L17" s="41" t="n"/>
+      <c r="M17" s="41" t="n"/>
+      <c r="N17" s="41" t="n"/>
+      <c r="O17" s="44">
         <f>IF(B17="","",IF(K17&lt;&gt;"","Destruido",IF(TODAY()&gt;EDATE(B17,12),"⚠ PENDIENTE DE DESTRUIR","En custodia")))</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="40" t="n"/>
-      <c r="B18" s="41" t="n"/>
-      <c r="C18" s="40" t="n"/>
-      <c r="D18" s="40" t="n"/>
-      <c r="E18" s="40" t="n"/>
-      <c r="F18" s="40" t="n"/>
-      <c r="G18" s="40" t="n"/>
-      <c r="H18" s="40" t="n"/>
-      <c r="I18" s="41" t="n"/>
-      <c r="J18" s="42">
+      <c r="A18" s="41" t="n"/>
+      <c r="B18" s="42" t="n"/>
+      <c r="C18" s="41" t="n"/>
+      <c r="D18" s="41" t="n"/>
+      <c r="E18" s="41" t="n"/>
+      <c r="F18" s="41" t="n"/>
+      <c r="G18" s="41" t="n"/>
+      <c r="H18" s="41" t="n"/>
+      <c r="I18" s="42" t="n"/>
+      <c r="J18" s="43">
         <f>IF(B18="","",EDATE(B18,12))</f>
         <v/>
       </c>
-      <c r="K18" s="41" t="n"/>
-      <c r="L18" s="40" t="n"/>
-      <c r="M18" s="40" t="n"/>
-      <c r="N18" s="40" t="n"/>
-      <c r="O18" s="43">
+      <c r="K18" s="42" t="n"/>
+      <c r="L18" s="41" t="n"/>
+      <c r="M18" s="41" t="n"/>
+      <c r="N18" s="41" t="n"/>
+      <c r="O18" s="44">
         <f>IF(B18="","",IF(K18&lt;&gt;"","Destruido",IF(TODAY()&gt;EDATE(B18,12),"⚠ PENDIENTE DE DESTRUIR","En custodia")))</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="40" t="n"/>
-      <c r="B19" s="41" t="n"/>
-      <c r="C19" s="40" t="n"/>
-      <c r="D19" s="40" t="n"/>
-      <c r="E19" s="40" t="n"/>
-      <c r="F19" s="40" t="n"/>
-      <c r="G19" s="40" t="n"/>
-      <c r="H19" s="40" t="n"/>
-      <c r="I19" s="41" t="n"/>
-      <c r="J19" s="42">
+      <c r="A19" s="41" t="n"/>
+      <c r="B19" s="42" t="n"/>
+      <c r="C19" s="41" t="n"/>
+      <c r="D19" s="41" t="n"/>
+      <c r="E19" s="41" t="n"/>
+      <c r="F19" s="41" t="n"/>
+      <c r="G19" s="41" t="n"/>
+      <c r="H19" s="41" t="n"/>
+      <c r="I19" s="42" t="n"/>
+      <c r="J19" s="43">
         <f>IF(B19="","",EDATE(B19,12))</f>
         <v/>
       </c>
-      <c r="K19" s="41" t="n"/>
-      <c r="L19" s="40" t="n"/>
-      <c r="M19" s="40" t="n"/>
-      <c r="N19" s="40" t="n"/>
-      <c r="O19" s="43">
+      <c r="K19" s="42" t="n"/>
+      <c r="L19" s="41" t="n"/>
+      <c r="M19" s="41" t="n"/>
+      <c r="N19" s="41" t="n"/>
+      <c r="O19" s="44">
         <f>IF(B19="","",IF(K19&lt;&gt;"","Destruido",IF(TODAY()&gt;EDATE(B19,12),"⚠ PENDIENTE DE DESTRUIR","En custodia")))</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="40" t="n"/>
-      <c r="B20" s="41" t="n"/>
-      <c r="C20" s="40" t="n"/>
-      <c r="D20" s="40" t="n"/>
-      <c r="E20" s="40" t="n"/>
-      <c r="F20" s="40" t="n"/>
-      <c r="G20" s="40" t="n"/>
-      <c r="H20" s="40" t="n"/>
-      <c r="I20" s="41" t="n"/>
-      <c r="J20" s="42">
+      <c r="A20" s="41" t="n"/>
+      <c r="B20" s="42" t="n"/>
+      <c r="C20" s="41" t="n"/>
+      <c r="D20" s="41" t="n"/>
+      <c r="E20" s="41" t="n"/>
+      <c r="F20" s="41" t="n"/>
+      <c r="G20" s="41" t="n"/>
+      <c r="H20" s="41" t="n"/>
+      <c r="I20" s="42" t="n"/>
+      <c r="J20" s="43">
         <f>IF(B20="","",EDATE(B20,12))</f>
         <v/>
       </c>
-      <c r="K20" s="41" t="n"/>
-      <c r="L20" s="40" t="n"/>
-      <c r="M20" s="40" t="n"/>
-      <c r="N20" s="40" t="n"/>
-      <c r="O20" s="43">
+      <c r="K20" s="42" t="n"/>
+      <c r="L20" s="41" t="n"/>
+      <c r="M20" s="41" t="n"/>
+      <c r="N20" s="41" t="n"/>
+      <c r="O20" s="44">
         <f>IF(B20="","",IF(K20&lt;&gt;"","Destruido",IF(TODAY()&gt;EDATE(B20,12),"⚠ PENDIENTE DE DESTRUIR","En custodia")))</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="40" t="n"/>
-      <c r="B21" s="41" t="n"/>
-      <c r="C21" s="40" t="n"/>
-      <c r="D21" s="40" t="n"/>
-      <c r="E21" s="40" t="n"/>
-      <c r="F21" s="40" t="n"/>
-      <c r="G21" s="40" t="n"/>
-      <c r="H21" s="40" t="n"/>
-      <c r="I21" s="41" t="n"/>
-      <c r="J21" s="42">
+      <c r="A21" s="41" t="n"/>
+      <c r="B21" s="42" t="n"/>
+      <c r="C21" s="41" t="n"/>
+      <c r="D21" s="41" t="n"/>
+      <c r="E21" s="41" t="n"/>
+      <c r="F21" s="41" t="n"/>
+      <c r="G21" s="41" t="n"/>
+      <c r="H21" s="41" t="n"/>
+      <c r="I21" s="42" t="n"/>
+      <c r="J21" s="43">
         <f>IF(B21="","",EDATE(B21,12))</f>
         <v/>
       </c>
-      <c r="K21" s="41" t="n"/>
-      <c r="L21" s="40" t="n"/>
-      <c r="M21" s="40" t="n"/>
-      <c r="N21" s="40" t="n"/>
-      <c r="O21" s="43">
+      <c r="K21" s="42" t="n"/>
+      <c r="L21" s="41" t="n"/>
+      <c r="M21" s="41" t="n"/>
+      <c r="N21" s="41" t="n"/>
+      <c r="O21" s="44">
         <f>IF(B21="","",IF(K21&lt;&gt;"","Destruido",IF(TODAY()&gt;EDATE(B21,12),"⚠ PENDIENTE DE DESTRUIR","En custodia")))</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="40" t="n"/>
-      <c r="B22" s="41" t="n"/>
-      <c r="C22" s="40" t="n"/>
-      <c r="D22" s="40" t="n"/>
-      <c r="E22" s="40" t="n"/>
-      <c r="F22" s="40" t="n"/>
-      <c r="G22" s="40" t="n"/>
-      <c r="H22" s="40" t="n"/>
-      <c r="I22" s="41" t="n"/>
-      <c r="J22" s="42">
+      <c r="A22" s="41" t="n"/>
+      <c r="B22" s="42" t="n"/>
+      <c r="C22" s="41" t="n"/>
+      <c r="D22" s="41" t="n"/>
+      <c r="E22" s="41" t="n"/>
+      <c r="F22" s="41" t="n"/>
+      <c r="G22" s="41" t="n"/>
+      <c r="H22" s="41" t="n"/>
+      <c r="I22" s="42" t="n"/>
+      <c r="J22" s="43">
         <f>IF(B22="","",EDATE(B22,12))</f>
         <v/>
       </c>
-      <c r="K22" s="41" t="n"/>
-      <c r="L22" s="40" t="n"/>
-      <c r="M22" s="40" t="n"/>
-      <c r="N22" s="40" t="n"/>
-      <c r="O22" s="43">
+      <c r="K22" s="42" t="n"/>
+      <c r="L22" s="41" t="n"/>
+      <c r="M22" s="41" t="n"/>
+      <c r="N22" s="41" t="n"/>
+      <c r="O22" s="44">
         <f>IF(B22="","",IF(K22&lt;&gt;"","Destruido",IF(TODAY()&gt;EDATE(B22,12),"⚠ PENDIENTE DE DESTRUIR","En custodia")))</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="40" t="n"/>
-      <c r="B23" s="41" t="n"/>
-      <c r="C23" s="40" t="n"/>
-      <c r="D23" s="40" t="n"/>
-      <c r="E23" s="40" t="n"/>
-      <c r="F23" s="40" t="n"/>
-      <c r="G23" s="40" t="n"/>
-      <c r="H23" s="40" t="n"/>
-      <c r="I23" s="41" t="n"/>
-      <c r="J23" s="42">
+      <c r="A23" s="41" t="n"/>
+      <c r="B23" s="42" t="n"/>
+      <c r="C23" s="41" t="n"/>
+      <c r="D23" s="41" t="n"/>
+      <c r="E23" s="41" t="n"/>
+      <c r="F23" s="41" t="n"/>
+      <c r="G23" s="41" t="n"/>
+      <c r="H23" s="41" t="n"/>
+      <c r="I23" s="42" t="n"/>
+      <c r="J23" s="43">
         <f>IF(B23="","",EDATE(B23,12))</f>
         <v/>
       </c>
-      <c r="K23" s="41" t="n"/>
-      <c r="L23" s="40" t="n"/>
-      <c r="M23" s="40" t="n"/>
-      <c r="N23" s="40" t="n"/>
-      <c r="O23" s="43">
+      <c r="K23" s="42" t="n"/>
+      <c r="L23" s="41" t="n"/>
+      <c r="M23" s="41" t="n"/>
+      <c r="N23" s="41" t="n"/>
+      <c r="O23" s="44">
         <f>IF(B23="","",IF(K23&lt;&gt;"","Destruido",IF(TODAY()&gt;EDATE(B23,12),"⚠ PENDIENTE DE DESTRUIR","En custodia")))</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="40" t="n"/>
-      <c r="B24" s="41" t="n"/>
-      <c r="C24" s="40" t="n"/>
-      <c r="D24" s="40" t="n"/>
-      <c r="E24" s="40" t="n"/>
-      <c r="F24" s="40" t="n"/>
-      <c r="G24" s="40" t="n"/>
-      <c r="H24" s="40" t="n"/>
-      <c r="I24" s="41" t="n"/>
-      <c r="J24" s="42">
+      <c r="A24" s="41" t="n"/>
+      <c r="B24" s="42" t="n"/>
+      <c r="C24" s="41" t="n"/>
+      <c r="D24" s="41" t="n"/>
+      <c r="E24" s="41" t="n"/>
+      <c r="F24" s="41" t="n"/>
+      <c r="G24" s="41" t="n"/>
+      <c r="H24" s="41" t="n"/>
+      <c r="I24" s="42" t="n"/>
+      <c r="J24" s="43">
         <f>IF(B24="","",EDATE(B24,12))</f>
         <v/>
       </c>
-      <c r="K24" s="41" t="n"/>
-      <c r="L24" s="40" t="n"/>
-      <c r="M24" s="40" t="n"/>
-      <c r="N24" s="40" t="n"/>
-      <c r="O24" s="43">
+      <c r="K24" s="42" t="n"/>
+      <c r="L24" s="41" t="n"/>
+      <c r="M24" s="41" t="n"/>
+      <c r="N24" s="41" t="n"/>
+      <c r="O24" s="44">
         <f>IF(B24="","",IF(K24&lt;&gt;"","Destruido",IF(TODAY()&gt;EDATE(B24,12),"⚠ PENDIENTE DE DESTRUIR","En custodia")))</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="40" t="n"/>
-      <c r="B25" s="41" t="n"/>
-      <c r="C25" s="40" t="n"/>
-      <c r="D25" s="40" t="n"/>
-      <c r="E25" s="40" t="n"/>
-      <c r="F25" s="40" t="n"/>
-      <c r="G25" s="40" t="n"/>
-      <c r="H25" s="40" t="n"/>
-      <c r="I25" s="41" t="n"/>
-      <c r="J25" s="42">
+      <c r="A25" s="41" t="n"/>
+      <c r="B25" s="42" t="n"/>
+      <c r="C25" s="41" t="n"/>
+      <c r="D25" s="41" t="n"/>
+      <c r="E25" s="41" t="n"/>
+      <c r="F25" s="41" t="n"/>
+      <c r="G25" s="41" t="n"/>
+      <c r="H25" s="41" t="n"/>
+      <c r="I25" s="42" t="n"/>
+      <c r="J25" s="43">
         <f>IF(B25="","",EDATE(B25,12))</f>
         <v/>
       </c>
-      <c r="K25" s="41" t="n"/>
-      <c r="L25" s="40" t="n"/>
-      <c r="M25" s="40" t="n"/>
-      <c r="N25" s="40" t="n"/>
-      <c r="O25" s="43">
+      <c r="K25" s="42" t="n"/>
+      <c r="L25" s="41" t="n"/>
+      <c r="M25" s="41" t="n"/>
+      <c r="N25" s="41" t="n"/>
+      <c r="O25" s="44">
         <f>IF(B25="","",IF(K25&lt;&gt;"","Destruido",IF(TODAY()&gt;EDATE(B25,12),"⚠ PENDIENTE DE DESTRUIR","En custodia")))</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="40" t="n"/>
-      <c r="B26" s="41" t="n"/>
-      <c r="C26" s="40" t="n"/>
-      <c r="D26" s="40" t="n"/>
-      <c r="E26" s="40" t="n"/>
-      <c r="F26" s="40" t="n"/>
-      <c r="G26" s="40" t="n"/>
-      <c r="H26" s="40" t="n"/>
-      <c r="I26" s="41" t="n"/>
-      <c r="J26" s="42">
+      <c r="A26" s="41" t="n"/>
+      <c r="B26" s="42" t="n"/>
+      <c r="C26" s="41" t="n"/>
+      <c r="D26" s="41" t="n"/>
+      <c r="E26" s="41" t="n"/>
+      <c r="F26" s="41" t="n"/>
+      <c r="G26" s="41" t="n"/>
+      <c r="H26" s="41" t="n"/>
+      <c r="I26" s="42" t="n"/>
+      <c r="J26" s="43">
         <f>IF(B26="","",EDATE(B26,12))</f>
         <v/>
       </c>
-      <c r="K26" s="41" t="n"/>
-      <c r="L26" s="40" t="n"/>
-      <c r="M26" s="40" t="n"/>
-      <c r="N26" s="40" t="n"/>
-      <c r="O26" s="43">
+      <c r="K26" s="42" t="n"/>
+      <c r="L26" s="41" t="n"/>
+      <c r="M26" s="41" t="n"/>
+      <c r="N26" s="41" t="n"/>
+      <c r="O26" s="44">
         <f>IF(B26="","",IF(K26&lt;&gt;"","Destruido",IF(TODAY()&gt;EDATE(B26,12),"⚠ PENDIENTE DE DESTRUIR","En custodia")))</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="40" t="n"/>
-      <c r="B27" s="41" t="n"/>
-      <c r="C27" s="40" t="n"/>
-      <c r="D27" s="40" t="n"/>
-      <c r="E27" s="40" t="n"/>
-      <c r="F27" s="40" t="n"/>
-      <c r="G27" s="40" t="n"/>
-      <c r="H27" s="40" t="n"/>
-      <c r="I27" s="41" t="n"/>
-      <c r="J27" s="42">
+      <c r="A27" s="41" t="n"/>
+      <c r="B27" s="42" t="n"/>
+      <c r="C27" s="41" t="n"/>
+      <c r="D27" s="41" t="n"/>
+      <c r="E27" s="41" t="n"/>
+      <c r="F27" s="41" t="n"/>
+      <c r="G27" s="41" t="n"/>
+      <c r="H27" s="41" t="n"/>
+      <c r="I27" s="42" t="n"/>
+      <c r="J27" s="43">
         <f>IF(B27="","",EDATE(B27,12))</f>
         <v/>
       </c>
-      <c r="K27" s="41" t="n"/>
-      <c r="L27" s="40" t="n"/>
-      <c r="M27" s="40" t="n"/>
-      <c r="N27" s="40" t="n"/>
-      <c r="O27" s="43">
+      <c r="K27" s="42" t="n"/>
+      <c r="L27" s="41" t="n"/>
+      <c r="M27" s="41" t="n"/>
+      <c r="N27" s="41" t="n"/>
+      <c r="O27" s="44">
         <f>IF(B27="","",IF(K27&lt;&gt;"","Destruido",IF(TODAY()&gt;EDATE(B27,12),"⚠ PENDIENTE DE DESTRUIR","En custodia")))</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="40" t="n"/>
-      <c r="B28" s="41" t="n"/>
-      <c r="C28" s="40" t="n"/>
-      <c r="D28" s="40" t="n"/>
-      <c r="E28" s="40" t="n"/>
-      <c r="F28" s="40" t="n"/>
-      <c r="G28" s="40" t="n"/>
-      <c r="H28" s="40" t="n"/>
-      <c r="I28" s="41" t="n"/>
-      <c r="J28" s="42">
+      <c r="A28" s="41" t="n"/>
+      <c r="B28" s="42" t="n"/>
+      <c r="C28" s="41" t="n"/>
+      <c r="D28" s="41" t="n"/>
+      <c r="E28" s="41" t="n"/>
+      <c r="F28" s="41" t="n"/>
+      <c r="G28" s="41" t="n"/>
+      <c r="H28" s="41" t="n"/>
+      <c r="I28" s="42" t="n"/>
+      <c r="J28" s="43">
         <f>IF(B28="","",EDATE(B28,12))</f>
         <v/>
       </c>
-      <c r="K28" s="41" t="n"/>
-      <c r="L28" s="40" t="n"/>
-      <c r="M28" s="40" t="n"/>
-      <c r="N28" s="40" t="n"/>
-      <c r="O28" s="43">
+      <c r="K28" s="42" t="n"/>
+      <c r="L28" s="41" t="n"/>
+      <c r="M28" s="41" t="n"/>
+      <c r="N28" s="41" t="n"/>
+      <c r="O28" s="44">
         <f>IF(B28="","",IF(K28&lt;&gt;"","Destruido",IF(TODAY()&gt;EDATE(B28,12),"⚠ PENDIENTE DE DESTRUIR","En custodia")))</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="40" t="n"/>
-      <c r="B29" s="41" t="n"/>
-      <c r="C29" s="40" t="n"/>
-      <c r="D29" s="40" t="n"/>
-      <c r="E29" s="40" t="n"/>
-      <c r="F29" s="40" t="n"/>
-      <c r="G29" s="40" t="n"/>
-      <c r="H29" s="40" t="n"/>
-      <c r="I29" s="41" t="n"/>
-      <c r="J29" s="42">
+      <c r="A29" s="41" t="n"/>
+      <c r="B29" s="42" t="n"/>
+      <c r="C29" s="41" t="n"/>
+      <c r="D29" s="41" t="n"/>
+      <c r="E29" s="41" t="n"/>
+      <c r="F29" s="41" t="n"/>
+      <c r="G29" s="41" t="n"/>
+      <c r="H29" s="41" t="n"/>
+      <c r="I29" s="42" t="n"/>
+      <c r="J29" s="43">
         <f>IF(B29="","",EDATE(B29,12))</f>
         <v/>
       </c>
-      <c r="K29" s="41" t="n"/>
-      <c r="L29" s="40" t="n"/>
-      <c r="M29" s="40" t="n"/>
-      <c r="N29" s="40" t="n"/>
-      <c r="O29" s="43">
+      <c r="K29" s="42" t="n"/>
+      <c r="L29" s="41" t="n"/>
+      <c r="M29" s="41" t="n"/>
+      <c r="N29" s="41" t="n"/>
+      <c r="O29" s="44">
         <f>IF(B29="","",IF(K29&lt;&gt;"","Destruido",IF(TODAY()&gt;EDATE(B29,12),"⚠ PENDIENTE DE DESTRUIR","En custodia")))</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="40" t="n"/>
-      <c r="B30" s="41" t="n"/>
-      <c r="C30" s="40" t="n"/>
-      <c r="D30" s="40" t="n"/>
-      <c r="E30" s="40" t="n"/>
-      <c r="F30" s="40" t="n"/>
-      <c r="G30" s="40" t="n"/>
-      <c r="H30" s="40" t="n"/>
-      <c r="I30" s="41" t="n"/>
-      <c r="J30" s="42">
+      <c r="A30" s="41" t="n"/>
+      <c r="B30" s="42" t="n"/>
+      <c r="C30" s="41" t="n"/>
+      <c r="D30" s="41" t="n"/>
+      <c r="E30" s="41" t="n"/>
+      <c r="F30" s="41" t="n"/>
+      <c r="G30" s="41" t="n"/>
+      <c r="H30" s="41" t="n"/>
+      <c r="I30" s="42" t="n"/>
+      <c r="J30" s="43">
         <f>IF(B30="","",EDATE(B30,12))</f>
         <v/>
       </c>
-      <c r="K30" s="41" t="n"/>
-      <c r="L30" s="40" t="n"/>
-      <c r="M30" s="40" t="n"/>
-      <c r="N30" s="40" t="n"/>
-      <c r="O30" s="43">
+      <c r="K30" s="42" t="n"/>
+      <c r="L30" s="41" t="n"/>
+      <c r="M30" s="41" t="n"/>
+      <c r="N30" s="41" t="n"/>
+      <c r="O30" s="44">
         <f>IF(B30="","",IF(K30&lt;&gt;"","Destruido",IF(TODAY()&gt;EDATE(B30,12),"⚠ PENDIENTE DE DESTRUIR","En custodia")))</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="40" t="n"/>
-      <c r="B31" s="41" t="n"/>
-      <c r="C31" s="40" t="n"/>
-      <c r="D31" s="40" t="n"/>
-      <c r="E31" s="40" t="n"/>
-      <c r="F31" s="40" t="n"/>
-      <c r="G31" s="40" t="n"/>
-      <c r="H31" s="40" t="n"/>
-      <c r="I31" s="41" t="n"/>
-      <c r="J31" s="42">
+      <c r="A31" s="41" t="n"/>
+      <c r="B31" s="42" t="n"/>
+      <c r="C31" s="41" t="n"/>
+      <c r="D31" s="41" t="n"/>
+      <c r="E31" s="41" t="n"/>
+      <c r="F31" s="41" t="n"/>
+      <c r="G31" s="41" t="n"/>
+      <c r="H31" s="41" t="n"/>
+      <c r="I31" s="42" t="n"/>
+      <c r="J31" s="43">
         <f>IF(B31="","",EDATE(B31,12))</f>
         <v/>
       </c>
-      <c r="K31" s="41" t="n"/>
-      <c r="L31" s="40" t="n"/>
-      <c r="M31" s="40" t="n"/>
-      <c r="N31" s="40" t="n"/>
-      <c r="O31" s="43">
+      <c r="K31" s="42" t="n"/>
+      <c r="L31" s="41" t="n"/>
+      <c r="M31" s="41" t="n"/>
+      <c r="N31" s="41" t="n"/>
+      <c r="O31" s="44">
         <f>IF(B31="","",IF(K31&lt;&gt;"","Destruido",IF(TODAY()&gt;EDATE(B31,12),"⚠ PENDIENTE DE DESTRUIR","En custodia")))</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="40" t="n"/>
-      <c r="B32" s="41" t="n"/>
-      <c r="C32" s="40" t="n"/>
-      <c r="D32" s="40" t="n"/>
-      <c r="E32" s="40" t="n"/>
-      <c r="F32" s="40" t="n"/>
-      <c r="G32" s="40" t="n"/>
-      <c r="H32" s="40" t="n"/>
-      <c r="I32" s="41" t="n"/>
-      <c r="J32" s="42">
+      <c r="A32" s="41" t="n"/>
+      <c r="B32" s="42" t="n"/>
+      <c r="C32" s="41" t="n"/>
+      <c r="D32" s="41" t="n"/>
+      <c r="E32" s="41" t="n"/>
+      <c r="F32" s="41" t="n"/>
+      <c r="G32" s="41" t="n"/>
+      <c r="H32" s="41" t="n"/>
+      <c r="I32" s="42" t="n"/>
+      <c r="J32" s="43">
         <f>IF(B32="","",EDATE(B32,12))</f>
         <v/>
       </c>
-      <c r="K32" s="41" t="n"/>
-      <c r="L32" s="40" t="n"/>
-      <c r="M32" s="40" t="n"/>
-      <c r="N32" s="40" t="n"/>
-      <c r="O32" s="43">
+      <c r="K32" s="42" t="n"/>
+      <c r="L32" s="41" t="n"/>
+      <c r="M32" s="41" t="n"/>
+      <c r="N32" s="41" t="n"/>
+      <c r="O32" s="44">
         <f>IF(B32="","",IF(K32&lt;&gt;"","Destruido",IF(TODAY()&gt;EDATE(B32,12),"⚠ PENDIENTE DE DESTRUIR","En custodia")))</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="40" t="n"/>
-      <c r="B33" s="41" t="n"/>
-      <c r="C33" s="40" t="n"/>
-      <c r="D33" s="40" t="n"/>
-      <c r="E33" s="40" t="n"/>
-      <c r="F33" s="40" t="n"/>
-      <c r="G33" s="40" t="n"/>
-      <c r="H33" s="40" t="n"/>
-      <c r="I33" s="41" t="n"/>
-      <c r="J33" s="42">
+      <c r="A33" s="41" t="n"/>
+      <c r="B33" s="42" t="n"/>
+      <c r="C33" s="41" t="n"/>
+      <c r="D33" s="41" t="n"/>
+      <c r="E33" s="41" t="n"/>
+      <c r="F33" s="41" t="n"/>
+      <c r="G33" s="41" t="n"/>
+      <c r="H33" s="41" t="n"/>
+      <c r="I33" s="42" t="n"/>
+      <c r="J33" s="43">
         <f>IF(B33="","",EDATE(B33,12))</f>
         <v/>
       </c>
-      <c r="K33" s="41" t="n"/>
-      <c r="L33" s="40" t="n"/>
-      <c r="M33" s="40" t="n"/>
-      <c r="N33" s="40" t="n"/>
-      <c r="O33" s="43">
+      <c r="K33" s="42" t="n"/>
+      <c r="L33" s="41" t="n"/>
+      <c r="M33" s="41" t="n"/>
+      <c r="N33" s="41" t="n"/>
+      <c r="O33" s="44">
         <f>IF(B33="","",IF(K33&lt;&gt;"","Destruido",IF(TODAY()&gt;EDATE(B33,12),"⚠ PENDIENTE DE DESTRUIR","En custodia")))</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="40" t="n"/>
-      <c r="B34" s="41" t="n"/>
-      <c r="C34" s="40" t="n"/>
-      <c r="D34" s="40" t="n"/>
-      <c r="E34" s="40" t="n"/>
-      <c r="F34" s="40" t="n"/>
-      <c r="G34" s="40" t="n"/>
-      <c r="H34" s="40" t="n"/>
-      <c r="I34" s="41" t="n"/>
-      <c r="J34" s="42">
+      <c r="A34" s="41" t="n"/>
+      <c r="B34" s="42" t="n"/>
+      <c r="C34" s="41" t="n"/>
+      <c r="D34" s="41" t="n"/>
+      <c r="E34" s="41" t="n"/>
+      <c r="F34" s="41" t="n"/>
+      <c r="G34" s="41" t="n"/>
+      <c r="H34" s="41" t="n"/>
+      <c r="I34" s="42" t="n"/>
+      <c r="J34" s="43">
         <f>IF(B34="","",EDATE(B34,12))</f>
         <v/>
       </c>
-      <c r="K34" s="41" t="n"/>
-      <c r="L34" s="40" t="n"/>
-      <c r="M34" s="40" t="n"/>
-      <c r="N34" s="40" t="n"/>
-      <c r="O34" s="43">
+      <c r="K34" s="42" t="n"/>
+      <c r="L34" s="41" t="n"/>
+      <c r="M34" s="41" t="n"/>
+      <c r="N34" s="41" t="n"/>
+      <c r="O34" s="44">
         <f>IF(B34="","",IF(K34&lt;&gt;"","Destruido",IF(TODAY()&gt;EDATE(B34,12),"⚠ PENDIENTE DE DESTRUIR","En custodia")))</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="40" t="n"/>
-      <c r="B35" s="41" t="n"/>
-      <c r="C35" s="40" t="n"/>
-      <c r="D35" s="40" t="n"/>
-      <c r="E35" s="40" t="n"/>
-      <c r="F35" s="40" t="n"/>
-      <c r="G35" s="40" t="n"/>
-      <c r="H35" s="40" t="n"/>
-      <c r="I35" s="41" t="n"/>
-      <c r="J35" s="42">
+      <c r="A35" s="41" t="n"/>
+      <c r="B35" s="42" t="n"/>
+      <c r="C35" s="41" t="n"/>
+      <c r="D35" s="41" t="n"/>
+      <c r="E35" s="41" t="n"/>
+      <c r="F35" s="41" t="n"/>
+      <c r="G35" s="41" t="n"/>
+      <c r="H35" s="41" t="n"/>
+      <c r="I35" s="42" t="n"/>
+      <c r="J35" s="43">
         <f>IF(B35="","",EDATE(B35,12))</f>
         <v/>
       </c>
-      <c r="K35" s="41" t="n"/>
-      <c r="L35" s="40" t="n"/>
-      <c r="M35" s="40" t="n"/>
-      <c r="N35" s="40" t="n"/>
-      <c r="O35" s="43">
+      <c r="K35" s="42" t="n"/>
+      <c r="L35" s="41" t="n"/>
+      <c r="M35" s="41" t="n"/>
+      <c r="N35" s="41" t="n"/>
+      <c r="O35" s="44">
         <f>IF(B35="","",IF(K35&lt;&gt;"","Destruido",IF(TODAY()&gt;EDATE(B35,12),"⚠ PENDIENTE DE DESTRUIR","En custodia")))</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="40" t="n"/>
-      <c r="B36" s="41" t="n"/>
-      <c r="C36" s="40" t="n"/>
-      <c r="D36" s="40" t="n"/>
-      <c r="E36" s="40" t="n"/>
-      <c r="F36" s="40" t="n"/>
-      <c r="G36" s="40" t="n"/>
-      <c r="H36" s="40" t="n"/>
-      <c r="I36" s="41" t="n"/>
-      <c r="J36" s="42">
+      <c r="A36" s="41" t="n"/>
+      <c r="B36" s="42" t="n"/>
+      <c r="C36" s="41" t="n"/>
+      <c r="D36" s="41" t="n"/>
+      <c r="E36" s="41" t="n"/>
+      <c r="F36" s="41" t="n"/>
+      <c r="G36" s="41" t="n"/>
+      <c r="H36" s="41" t="n"/>
+      <c r="I36" s="42" t="n"/>
+      <c r="J36" s="43">
         <f>IF(B36="","",EDATE(B36,12))</f>
         <v/>
       </c>
-      <c r="K36" s="41" t="n"/>
-      <c r="L36" s="40" t="n"/>
-      <c r="M36" s="40" t="n"/>
-      <c r="N36" s="40" t="n"/>
-      <c r="O36" s="43">
+      <c r="K36" s="42" t="n"/>
+      <c r="L36" s="41" t="n"/>
+      <c r="M36" s="41" t="n"/>
+      <c r="N36" s="41" t="n"/>
+      <c r="O36" s="44">
         <f>IF(B36="","",IF(K36&lt;&gt;"","Destruido",IF(TODAY()&gt;EDATE(B36,12),"⚠ PENDIENTE DE DESTRUIR","En custodia")))</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="40" t="n"/>
-      <c r="B37" s="41" t="n"/>
-      <c r="C37" s="40" t="n"/>
-      <c r="D37" s="40" t="n"/>
-      <c r="E37" s="40" t="n"/>
-      <c r="F37" s="40" t="n"/>
-      <c r="G37" s="40" t="n"/>
-      <c r="H37" s="40" t="n"/>
-      <c r="I37" s="41" t="n"/>
-      <c r="J37" s="42">
+      <c r="A37" s="41" t="n"/>
+      <c r="B37" s="42" t="n"/>
+      <c r="C37" s="41" t="n"/>
+      <c r="D37" s="41" t="n"/>
+      <c r="E37" s="41" t="n"/>
+      <c r="F37" s="41" t="n"/>
+      <c r="G37" s="41" t="n"/>
+      <c r="H37" s="41" t="n"/>
+      <c r="I37" s="42" t="n"/>
+      <c r="J37" s="43">
         <f>IF(B37="","",EDATE(B37,12))</f>
         <v/>
       </c>
-      <c r="K37" s="41" t="n"/>
-      <c r="L37" s="40" t="n"/>
-      <c r="M37" s="40" t="n"/>
-      <c r="N37" s="40" t="n"/>
-      <c r="O37" s="43">
+      <c r="K37" s="42" t="n"/>
+      <c r="L37" s="41" t="n"/>
+      <c r="M37" s="41" t="n"/>
+      <c r="N37" s="41" t="n"/>
+      <c r="O37" s="44">
         <f>IF(B37="","",IF(K37&lt;&gt;"","Destruido",IF(TODAY()&gt;EDATE(B37,12),"⚠ PENDIENTE DE DESTRUIR","En custodia")))</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="40" t="n"/>
-      <c r="B38" s="41" t="n"/>
-      <c r="C38" s="40" t="n"/>
-      <c r="D38" s="40" t="n"/>
-      <c r="E38" s="40" t="n"/>
-      <c r="F38" s="40" t="n"/>
-      <c r="G38" s="40" t="n"/>
-      <c r="H38" s="40" t="n"/>
-      <c r="I38" s="41" t="n"/>
-      <c r="J38" s="42">
+      <c r="A38" s="41" t="n"/>
+      <c r="B38" s="42" t="n"/>
+      <c r="C38" s="41" t="n"/>
+      <c r="D38" s="41" t="n"/>
+      <c r="E38" s="41" t="n"/>
+      <c r="F38" s="41" t="n"/>
+      <c r="G38" s="41" t="n"/>
+      <c r="H38" s="41" t="n"/>
+      <c r="I38" s="42" t="n"/>
+      <c r="J38" s="43">
         <f>IF(B38="","",EDATE(B38,12))</f>
         <v/>
       </c>
-      <c r="K38" s="41" t="n"/>
-      <c r="L38" s="40" t="n"/>
-      <c r="M38" s="40" t="n"/>
-      <c r="N38" s="40" t="n"/>
-      <c r="O38" s="43">
+      <c r="K38" s="42" t="n"/>
+      <c r="L38" s="41" t="n"/>
+      <c r="M38" s="41" t="n"/>
+      <c r="N38" s="41" t="n"/>
+      <c r="O38" s="44">
         <f>IF(B38="","",IF(K38&lt;&gt;"","Destruido",IF(TODAY()&gt;EDATE(B38,12),"⚠ PENDIENTE DE DESTRUIR","En custodia")))</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="40" t="n"/>
-      <c r="B39" s="41" t="n"/>
-      <c r="C39" s="40" t="n"/>
-      <c r="D39" s="40" t="n"/>
-      <c r="E39" s="40" t="n"/>
-      <c r="F39" s="40" t="n"/>
-      <c r="G39" s="40" t="n"/>
-      <c r="H39" s="40" t="n"/>
-      <c r="I39" s="41" t="n"/>
-      <c r="J39" s="42">
+      <c r="A39" s="41" t="n"/>
+      <c r="B39" s="42" t="n"/>
+      <c r="C39" s="41" t="n"/>
+      <c r="D39" s="41" t="n"/>
+      <c r="E39" s="41" t="n"/>
+      <c r="F39" s="41" t="n"/>
+      <c r="G39" s="41" t="n"/>
+      <c r="H39" s="41" t="n"/>
+      <c r="I39" s="42" t="n"/>
+      <c r="J39" s="43">
         <f>IF(B39="","",EDATE(B39,12))</f>
         <v/>
       </c>
-      <c r="K39" s="41" t="n"/>
-      <c r="L39" s="40" t="n"/>
-      <c r="M39" s="40" t="n"/>
-      <c r="N39" s="40" t="n"/>
-      <c r="O39" s="43">
+      <c r="K39" s="42" t="n"/>
+      <c r="L39" s="41" t="n"/>
+      <c r="M39" s="41" t="n"/>
+      <c r="N39" s="41" t="n"/>
+      <c r="O39" s="44">
         <f>IF(B39="","",IF(K39&lt;&gt;"","Destruido",IF(TODAY()&gt;EDATE(B39,12),"⚠ PENDIENTE DE DESTRUIR","En custodia")))</f>
         <v/>
       </c>
@@ -4319,7 +4324,7 @@
           <t>Trámite Generalitat (petició genèrica)</t>
         </is>
       </c>
-      <c r="B30" s="44" t="inlineStr">
+      <c r="B30" s="45" t="inlineStr">
         <is>
           <t>https://web.gencat.cat/ca/tramits/tramits-temes/Peticio-generica</t>
         </is>
@@ -4331,7 +4336,7 @@
           <t>Trámite Generalitat (formulario OVT)</t>
         </is>
       </c>
-      <c r="B31" s="44" t="inlineStr">
+      <c r="B31" s="45" t="inlineStr">
         <is>
           <t>https://ovt.gencat.cat/gsitgf/AppJava/traint/renderitzar.do?reqCode=inicial&amp;set-locale=ca_ES&amp;idioma=ca_ES&amp;idServei=ING001SOLC&amp;urlRetorn=https%3A%2F%2Fweb.gencat.cat%2Fca%2Ftramits%2Ftramits-temes%2FPeticio-generica%3Fmoda%3D1&amp;tpst=ae56fd5821cffc7f4784ac8db0c0e1a0</t>
         </is>
@@ -4417,7 +4422,7 @@
           <t>Txt_J_Informado</t>
         </is>
       </c>
-      <c r="B44" s="45" t="inlineStr">
+      <c r="B44" s="46" t="inlineStr">
         <is>
           <t xml:space="preserve">He sido informado por el centro técnico de tacógrafos de </t>
         </is>
@@ -4429,7 +4434,7 @@
           <t>Txt_J_Contrasena</t>
         </is>
       </c>
-      <c r="B45" s="45" t="inlineStr">
+      <c r="B45" s="46" t="inlineStr">
         <is>
           <t xml:space="preserve">con contraseña </t>
         </is>
@@ -4441,7 +4446,7 @@
           <t>Txt_J_Marca</t>
         </is>
       </c>
-      <c r="B46" s="45" t="inlineStr">
+      <c r="B46" s="46" t="inlineStr">
         <is>
           <t>, de que el tacógrafo marca:</t>
         </is>
@@ -4453,7 +4458,7 @@
           <t>Txt_En</t>
         </is>
       </c>
-      <c r="B47" s="45" t="inlineStr">
+      <c r="B47" s="46" t="inlineStr">
         <is>
           <t xml:space="preserve">En </t>
         </is>
@@ -4465,7 +4470,7 @@
           <t>Txt_A</t>
         </is>
       </c>
-      <c r="B48" s="45" t="inlineStr">
+      <c r="B48" s="46" t="inlineStr">
         <is>
           <t xml:space="preserve">, a </t>
         </is>
@@ -4477,7 +4482,7 @@
           <t>Txt_Sello</t>
         </is>
       </c>
-      <c r="B49" s="45" t="inlineStr">
+      <c r="B49" s="46" t="inlineStr">
         <is>
           <t xml:space="preserve">Sello </t>
         </is>
@@ -4489,7 +4494,7 @@
           <t>Txt_Entrega_Si</t>
         </is>
       </c>
-      <c r="B50" s="45" t="inlineStr">
+      <c r="B50" s="46" t="inlineStr">
         <is>
           <t>***Se entrega tacógrafo Averiado</t>
         </is>
@@ -4501,7 +4506,7 @@
           <t>Txt_Achatarrar_Si</t>
         </is>
       </c>
-      <c r="B51" s="45" t="inlineStr">
+      <c r="B51" s="46" t="inlineStr">
         <is>
           <t>***El tacógrafo se achatarrará</t>
         </is>
@@ -4513,7 +4518,7 @@
           <t>Txt_Fitxer</t>
         </is>
       </c>
-      <c r="B52" s="45" t="inlineStr">
+      <c r="B52" s="46" t="inlineStr">
         <is>
           <t xml:space="preserve"> Certificat de Intransferibilitat</t>
         </is>
@@ -4525,7 +4530,7 @@
           <t>Txt_Confid</t>
         </is>
       </c>
-      <c r="B53" s="45" t="inlineStr">
+      <c r="B53" s="46" t="inlineStr">
         <is>
           <t>Los datos contenidos en la memoria de la unidad intravehicular tienen carácter confidencial. El solicitante debe evaluar la confidencialidad de los datos transferidos para el procedimiento de remisión que elija. El centro técnico no será responsable de la violación de la confidencialidad de los datos durante su remisión (nota E del anexo II del Real decreto 125:2017).</t>
         </is>
@@ -4537,7 +4542,7 @@
           <t>Txt_Custodia</t>
         </is>
       </c>
-      <c r="B54" s="45" t="inlineStr">
+      <c r="B54" s="46" t="inlineStr">
         <is>
           <t>Los datos recuperados de la unidad instalada en el vehículo se guardarán en el centro técnico durante un año desde la fecha de la transferencia. Una vez cumplido dicho plazo, los datos serán destruidos (nota F del anexo II del Real decreto 125:2017).</t>
         </is>
@@ -4549,7 +4554,7 @@
           <t>Txt_Titularidad</t>
         </is>
       </c>
-      <c r="B55" s="45" t="inlineStr">
+      <c r="B55" s="46" t="inlineStr">
         <is>
           <t>Se ha presentado al centro técnico documento que avala la titularidad de los datos por parte de la empresa de transportes, verificado y archivado por el centro (nota D del anexo II del Real decreto 125:2017).</t>
         </is>
@@ -4561,7 +4566,7 @@
           <t>Txt_Cat_1</t>
         </is>
       </c>
-      <c r="B56" s="45" t="inlineStr">
+      <c r="B56" s="46" t="inlineStr">
         <is>
           <t xml:space="preserve">En compliment del requisit expressat en la disposició addicional primera, apartat 10, del Reial decret 125: 2017, els remetem còpia del certificat de intransferibilitat corresponent a la substitució del tacògraf: Model: </t>
         </is>
@@ -4573,7 +4578,7 @@
           <t>Txt_Cat_2</t>
         </is>
       </c>
-      <c r="B57" s="45" t="inlineStr">
+      <c r="B57" s="46" t="inlineStr">
         <is>
           <t xml:space="preserve">, Nº de Sèrie: </t>
         </is>
@@ -4585,7 +4590,7 @@
           <t>Txt_Cat_3</t>
         </is>
       </c>
-      <c r="B58" s="45" t="inlineStr">
+      <c r="B58" s="46" t="inlineStr">
         <is>
           <t xml:space="preserve">, muntat en el vehicle: </t>
         </is>
@@ -4597,7 +4602,7 @@
           <t>Txt_Cat_4</t>
         </is>
       </c>
-      <c r="B59" s="45" t="inlineStr">
+      <c r="B59" s="46" t="inlineStr">
         <is>
           <t xml:space="preserve">, Nº d'informe / certificat: </t>
         </is>
@@ -4609,7 +4614,7 @@
           <t>Txt_Cat_5</t>
         </is>
       </c>
-      <c r="B60" s="45" t="inlineStr">
+      <c r="B60" s="46" t="inlineStr">
         <is>
           <t xml:space="preserve">, Data Informe: </t>
         </is>
@@ -4621,7 +4626,7 @@
           <t>Txt_Cat_6</t>
         </is>
       </c>
-      <c r="B61" s="45" t="inlineStr">
+      <c r="B61" s="46" t="inlineStr">
         <is>
           <t>. Sol·licito que es doni el tràmit acceptat.</t>
         </is>

</xml_diff>

<commit_message>
fix(tacografos): separa autorizante de receptor y corrige la cita del RD 125/2017
El justificante lo firma quien autoriza la descarga; el acuse lo firma quien
recibe el certificado. El original ya los trataba como personas distintas
(K3/M3 frente a I9/I10), asi que vuelven a ser campos propios, sin relleno
automatico entre ellos.

Ademas se corrigen las ocho apariciones de "Real decreto 125:2017" y
"Reial decret 125: 2017": la referencia correcta lleva barra.

228 formulas, 0 errores.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TAp9Dxq8XWBh75W4jtVJj4
</commit_message>
<xml_diff>
--- a/docs/plantillas/TACOGRAFOS_documentacion.xlsx
+++ b/docs/plantillas/TACOGRAFOS_documentacion.xlsx
@@ -90,8 +90,10 @@
     <definedName name="Dat_Enviados">'DATOS'!$B$40</definedName>
     <definedName name="Dat_FechaEnvio">'DATOS'!$B$41</definedName>
     <definedName name="Dat_Modalidad">'DATOS'!$B$43</definedName>
-    <definedName name="Dat_EntregaAparato">'DATOS'!$B$45</definedName>
-    <definedName name="Dat_Achatarrar">'DATOS'!$B$46</definedName>
+    <definedName name="Dat_NombreReceptor">'DATOS'!$B$45</definedName>
+    <definedName name="Dat_DniReceptor">'DATOS'!$B$46</definedName>
+    <definedName name="Dat_EntregaAparato">'DATOS'!$B$48</definedName>
+    <definedName name="Dat_Achatarrar">'DATOS'!$B$49</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'JUSTIFICANTE TRANSFERENCIA'!$B$1:$H$30</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'ANEXO II RD 125-2017'!$A$1:$G$48</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'INTRANSFERIBILIDAD CLIENTE'!$A$1:$G$52</definedName>
@@ -765,7 +767,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D49"/>
+  <dimension ref="A1:D52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -788,7 +790,7 @@
         </is>
       </c>
       <c r="B2" s="3">
-        <f>IF(SUM(D5:D46)=0,"✔ Datos completos","⚠ Faltan "&amp;SUM(D5:D46)&amp;" campo(s) obligatorio(s)")</f>
+        <f>IF(SUM(D5:D49)=0,"✔ Datos completos","⚠ Faltan "&amp;SUM(D5:D49)&amp;" campo(s) obligatorio(s)")</f>
         <v/>
       </c>
     </row>
@@ -864,7 +866,7 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Nombre persona autorizada</t>
+          <t>Nombre de quien autoriza</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
@@ -884,7 +886,7 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>DNI / NIF</t>
+          <t>DNI / NIF de quien autoriza</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
@@ -1529,7 +1531,7 @@
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>TACÓGRAFO AVERIADO</t>
+          <t>PERSONA QUE RECIBE EL CERTIFICADO (acuse de intransferibilidad)</t>
         </is>
       </c>
       <c r="B44" s="5" t="n"/>
@@ -1538,12 +1540,12 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>Se entrega al cliente</t>
+          <t>Nombre de la persona receptora</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Marta Solé Vidal</t>
         </is>
       </c>
       <c r="C45" s="8">
@@ -1558,41 +1560,90 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>Se achatarrará (excluyente)</t>
-        </is>
-      </c>
-      <c r="B46" s="11">
-        <f>IF(B45="Sí","No",IF(B45="No","Sí",""))</f>
-        <v/>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>automático</t>
-        </is>
-      </c>
-      <c r="D46" t="n">
-        <v>0</v>
-      </c>
+          <t>DNI de la persona receptora</t>
+        </is>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>40123456X</t>
+        </is>
+      </c>
+      <c r="C46" s="8">
+        <f>IF(AND($B$28="Intransferibilidad",B46=""),"⚠ Obligatorio","")</f>
+        <v/>
+      </c>
+      <c r="D46" s="2">
+        <f>IF(C46&lt;&gt;"",1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>TACÓGRAFO AVERIADO</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n"/>
+      <c r="C47" s="5" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>Coherencia (UNE 66102:2025)</t>
-        </is>
-      </c>
-      <c r="B48" s="12">
-        <f>IF(AND($B$28="Transferencia correcta",OR(B36="No",B37="No")),"⚠ Marcado como transferencia correcta pero el anexo II dice que no se pudo transferir/descargar",IF(AND($B$28="Intransferibilidad",B36="Sí"),"⚠ Marcado como intransferibilidad pero el anexo II dice que sí era posible transferir",""))</f>
+          <t>Se entrega al cliente</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C48" s="8">
+        <f>IF(AND($B$28="Intransferibilidad",B48=""),"⚠ Obligatorio","")</f>
+        <v/>
+      </c>
+      <c r="D48" s="2">
+        <f>IF(C48&lt;&gt;"",1,0)</f>
         <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
+          <t>Se achatarrará (excluyente)</t>
+        </is>
+      </c>
+      <c r="B49" s="11">
+        <f>IF(B48="Sí","No",IF(B48="No","Sí",""))</f>
+        <v/>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>automático</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>Coherencia (UNE 66102:2025)</t>
+        </is>
+      </c>
+      <c r="B51" s="12">
+        <f>IF(AND($B$28="Transferencia correcta",OR(B36="No",B37="No")),"⚠ Marcado como transferencia correcta pero el anexo II dice que no se pudo transferir/descargar",IF(AND($B$28="Intransferibilidad",B36="Sí"),"⚠ Marcado como intransferibilidad pero el anexo II dice que sí era posible transferir",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
           <t>Destrucción de los archivos</t>
         </is>
       </c>
-      <c r="B49" s="2">
-        <f>IF(B39="","","Conservar hasta "&amp;RIGHT("0"&amp;DAY(EDATE(B39,12)),2)&amp;"/"&amp;RIGHT("0"&amp;MONTH(EDATE(B39,12)),2)&amp;"/"&amp;YEAR(EDATE(B39,12))&amp;" y destruir después (nota F, RD 125:2017)")</f>
+      <c r="B52" s="2">
+        <f>IF(B39="","","Conservar hasta "&amp;RIGHT("0"&amp;DAY(EDATE(B39,12)),2)&amp;"/"&amp;RIGHT("0"&amp;MONTH(EDATE(B39,12)),2)&amp;"/"&amp;YEAR(EDATE(B39,12))&amp;" y destruir después (nota F, RD 125/2017)")</f>
         <v/>
       </c>
     </row>
@@ -1600,10 +1651,10 @@
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <conditionalFormatting sqref="B2">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>SUM(D5:D46)&gt;0</formula>
+      <formula>SUM(D5:D49)&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:B46">
+  <conditionalFormatting sqref="B5:B49">
     <cfRule type="expression" priority="2" dxfId="0">
       <formula>$C5="⚠ Obligatorio"</formula>
     </cfRule>
@@ -1615,7 +1666,7 @@
     <dataValidation sqref="B43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=CONFIGURACION!$B$36:$B$39</formula1>
     </dataValidation>
-    <dataValidation sqref="B10 B21 B34 B35 B36 B37 B40 B45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B10 B21 B34 B35 B36 B37 B40 B48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=CONFIGURACION!$C$40:$C$41</formula1>
     </dataValidation>
     <dataValidation sqref="B20 B26 B27 B39 B41" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Fecha no válida" error="Introduce una fecha real en formato dd/mm/aaaa." type="date" operator="between">
@@ -1725,7 +1776,7 @@
     <row r="13" ht="60" customHeight="1">
       <c r="B13" s="16" t="inlineStr">
         <is>
-          <t>Doy la indicación, así mismo, de que los archivos de transferencia originados en la mencionada descarga sean entregados a la empresa propietaria del vehículo a través del medio indicado debajo, de entre las cuatro posibles opciones indicadas en el punto 6 de la disposición adicional primera del Real decreto 125:2017 (señálese la opción que proceda)</t>
+          <t>Doy la indicación, así mismo, de que los archivos de transferencia originados en la mencionada descarga sean entregados a la empresa propietaria del vehículo a través del medio indicado debajo, de entre las cuatro posibles opciones indicadas en el punto 6 de la disposición adicional primera del Real decreto 125/2017 (señálese la opción que proceda)</t>
         </is>
       </c>
     </row>
@@ -2568,7 +2619,7 @@
     <row r="16">
       <c r="A16" s="16" t="inlineStr">
         <is>
-          <t>En cumplimiento del requisito expresado en la disposición adicional primera, apartado 10, del Real decreto 125:2017, les remitimos copia del certificado de intransferibilidad correspondiente a la sustitución del tacógrafo:</t>
+          <t>En cumplimiento del requisito expresado en la disposición adicional primera, apartado 10, del Real decreto 125/2017, les remitimos copia del certificado de intransferibilidad correspondiente a la sustitución del tacógrafo:</t>
         </is>
       </c>
     </row>
@@ -2636,7 +2687,7 @@
         </is>
       </c>
       <c r="C27" s="13">
-        <f>IF('DATOS'!$B$8="","",'DATOS'!$B$8)</f>
+        <f>IF('DATOS'!$B$45="","",'DATOS'!$B$45)</f>
         <v/>
       </c>
     </row>
@@ -2647,7 +2698,7 @@
         </is>
       </c>
       <c r="C28" s="13">
-        <f>IF('DATOS'!$B$9="","",'DATOS'!$B$9)</f>
+        <f>IF('DATOS'!$B$46="","",'DATOS'!$B$46)</f>
         <v/>
       </c>
     </row>
@@ -2670,13 +2721,13 @@
     <row r="36"/>
     <row r="38">
       <c r="A38" s="13">
-        <f>IF('DATOS'!$B$45="Sí",'CONFIGURACION'!$B$50,"")</f>
+        <f>IF('DATOS'!$B$48="Sí",'CONFIGURACION'!$B$50,"")</f>
         <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="13">
-        <f>IF('DATOS'!$B$46="Sí",'CONFIGURACION'!$B$51,"")</f>
+        <f>IF('DATOS'!$B$49="Sí",'CONFIGURACION'!$B$51,"")</f>
         <v/>
       </c>
     </row>
@@ -2837,7 +2888,7 @@
     <row r="16">
       <c r="A16" s="16" t="inlineStr">
         <is>
-          <t>En cumplimiento del requisito expresado en la disposición adicional primera, apartado 10, del Real decreto 125:2017, les remitimos copia del certificado de intransferibilidad correspondiente a la sustitución del tacógrafo:</t>
+          <t>En cumplimiento del requisito expresado en la disposición adicional primera, apartado 10, del Real decreto 125/2017, les remitimos copia del certificado de intransferibilidad correspondiente a la sustitución del tacógrafo:</t>
         </is>
       </c>
     </row>
@@ -4532,7 +4583,7 @@
       </c>
       <c r="B53" s="46" t="inlineStr">
         <is>
-          <t>Los datos contenidos en la memoria de la unidad intravehicular tienen carácter confidencial. El solicitante debe evaluar la confidencialidad de los datos transferidos para el procedimiento de remisión que elija. El centro técnico no será responsable de la violación de la confidencialidad de los datos durante su remisión (nota E del anexo II del Real decreto 125:2017).</t>
+          <t>Los datos contenidos en la memoria de la unidad intravehicular tienen carácter confidencial. El solicitante debe evaluar la confidencialidad de los datos transferidos para el procedimiento de remisión que elija. El centro técnico no será responsable de la violación de la confidencialidad de los datos durante su remisión (nota E del anexo II del Real decreto 125/2017).</t>
         </is>
       </c>
     </row>
@@ -4544,7 +4595,7 @@
       </c>
       <c r="B54" s="46" t="inlineStr">
         <is>
-          <t>Los datos recuperados de la unidad instalada en el vehículo se guardarán en el centro técnico durante un año desde la fecha de la transferencia. Una vez cumplido dicho plazo, los datos serán destruidos (nota F del anexo II del Real decreto 125:2017).</t>
+          <t>Los datos recuperados de la unidad instalada en el vehículo se guardarán en el centro técnico durante un año desde la fecha de la transferencia. Una vez cumplido dicho plazo, los datos serán destruidos (nota F del anexo II del Real decreto 125/2017).</t>
         </is>
       </c>
     </row>
@@ -4556,7 +4607,7 @@
       </c>
       <c r="B55" s="46" t="inlineStr">
         <is>
-          <t>Se ha presentado al centro técnico documento que avala la titularidad de los datos por parte de la empresa de transportes, verificado y archivado por el centro (nota D del anexo II del Real decreto 125:2017).</t>
+          <t>Se ha presentado al centro técnico documento que avala la titularidad de los datos por parte de la empresa de transportes, verificado y archivado por el centro (nota D del anexo II del Real decreto 125/2017).</t>
         </is>
       </c>
     </row>
@@ -4568,7 +4619,7 @@
       </c>
       <c r="B56" s="46" t="inlineStr">
         <is>
-          <t xml:space="preserve">En compliment del requisit expressat en la disposició addicional primera, apartat 10, del Reial decret 125: 2017, els remetem còpia del certificat de intransferibilitat corresponent a la substitució del tacògraf: Model: </t>
+          <t xml:space="preserve">En compliment del requisit expressat en la disposició addicional primera, apartat 10, del Reial decret 125/2017, els remetem còpia del certificat de intransferibilitat corresponent a la substitució del tacògraf: Model: </t>
         </is>
       </c>
     </row>

</xml_diff>